<commit_message>
Track Volume 83-90 outputs + sync correction registry / GPO log / manifest
Snapshot of pipeline state after the most recent batch run:

- New Volume-83 through Volume-90 directories with published Excel +
  SME companion files (16 binary files, ~12 MB total).
- active_corrections.json: new approved entries discovered during the
  vols 83-90 runs.
- pending_corrections.json: same updates plus any still-open proposals.
- gpo_issue_log.xlsx: appended issue rows (per-volume dedup ensures no
  duplicate keys).
- run_manifest.json: per-volume provenance (hashes, output paths,
  corrections_applied, last_run timestamps).

The .gitignore was updated separately to allow processed_output/Volume-*/
to be tracked, replacing the earlier ignore-by-default rule.
</commit_message>
<xml_diff>
--- a/processed_output/gpo_issue_log.xlsx
+++ b/processed_output/gpo_issue_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -552,7 +552,6 @@
           <t>global</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>RESOLVED_BY_CODE</t>
@@ -2293,6 +2292,4967 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>83 Stat. 847</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>83</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>91 Session 1</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Unnumbered intro section and numbered Section 1 collapse to the same unique key</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>The unnumbered "That—" intro "section" element and the following "section" with "num" value 1 produce the same unique key; the extractor's null-fallback ordinal for the unnumbered intro should be distinct from real parsed section numbers in the same law.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>&lt;section class="inline"&gt;
+&lt;content class="inline"&gt;That— &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;Central Intelligence Agency Retirement Act of 1964 for Certain Employees, amendment.&lt;/p&gt;&lt;/sidenote&gt;&lt;/content&gt;
+&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content&gt;Section 211(a) of the Central Intelligence Agency Retirement Act of 1964 for Certain Employees, as amended (78 Stat. 1043; 50 U.S.C. 403 note), is further amended by striking out “Six and one-half per centum” in the first sentence and inserting “Seven per centum”.&lt;/content&gt;
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>46411-46561</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>84 Stat. 1204</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>84</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>91 Session 2</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Two distinct section tags both labeled Sec. 613 in the same pLaw</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>The second Sec. 613 (Citation of titles, short-title naming) should be Sec. 615 — it follows Sec. 613 (Relinquishment of legislative jurisdiction) and Sec. 614 (land exchange) and is misnumbered in the source XML.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;num value="613"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 613. &lt;/num&gt;...Chapter 139 of title 10, United States Code, is amended as follows:...Relinquishment of legislative jurisdiction...
+&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="614"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 614. &lt;/num&gt;...Army Secretary, land exchange, Va...Anheuser-Busch Company...
+&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="613"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 613. &lt;/num&gt;&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;Citation of titles.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;content class="inline"&gt;Titles I, II, III, IV, V, and VI of this Act may be cited as the “&lt;shortTitle role="act"&gt;Military Construction Authorization Act, 1911&lt;/shortTitle&gt;”.&lt;/content&gt;
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;title&gt;
+   &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>72847-72887</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>84 Stat. 1327</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>84</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>91 Session 2</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Two distinct section tags both labeled SEC. 401 in TITLE IV of the same pLaw</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>The second SEC. 401 (Discontinuance of Service) should be SEC. 404 — it follows the legitimate SEC. 401 (Assumption of Passenger Service), SEC. 402 (Facility and Service Agreements), and SEC. 403 (New Service) and is misnumbered in the source XML.</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;num value="401"&gt;SEC. 401. &lt;/num&gt;
+&lt;heading&gt;ASSUMPTION OF PASSENGER SERVICE BY THE CORPORATION; COMMENCEMENT OF OPERATIONS.&lt;/heading&gt;
+...
+&lt;/section&gt;
+&lt;section&gt;
+&lt;num value="402"&gt;SEC. 402. &lt;/num&gt;&lt;heading&gt;FACILITY AND SERVICE AGREEMENTS.&lt;/heading&gt;...
+&lt;/section&gt;
+&lt;section&gt;
+&lt;num value="403"&gt;SEC. 403. &lt;/num&gt;&lt;heading&gt;NEW SERVICE.&lt;/heading&gt;...
+&lt;/section&gt;
+&lt;section&gt;
+&lt;num value="401"&gt;SEC. 401. &lt;/num&gt;
+&lt;heading&gt;DISCONTINUANCE OF SERVICE.&lt;/heading&gt;
+...
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;title&gt;
+   &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>78996-79065</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>84 Stat. 1441</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>84</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>91 Session 2</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Two sibling appropriations elements share the identical heading "General Provisions" under different major appropriation parents (General Services Administration and National Aeronautics and Space Administration)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Heading-derived UniqueKey positions collapse because the extractor builds DivisionHeadingLevel from heading text alone and does not disambiguate sibling appropriations sharing heading text across different major parents. Same root cause as active correction #5 (sibling appropriations heading collapse, vol 78); the ordinal-disambiguation fix applies here as well.</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>&lt;appropriations level="major"&gt;&lt;heading&gt;GENERAL SERVICES ADMINISTRATION&lt;/heading&gt;
+...
+&lt;appropriations level="intermediate"&gt;&lt;heading&gt;General Provisions&lt;/heading&gt;
+&lt;content class="firstIndent1 fontsize10"&gt;...The appropriate appropriation or fund available to the General Services Administration shall be credited with...&lt;/content&gt;
+&lt;/appropriations&gt;
+&lt;/appropriations&gt;
+&lt;appropriations level="major"&gt;&lt;heading&gt;NATIONAL AERONAUTICS AND SPACE ADMINISTRATION&lt;/heading&gt;
+...
+&lt;appropriations level="intermediate"&gt;&lt;heading&gt;General Provisions&lt;/heading&gt;
+&lt;content class="firstIndent1 fontsize10"&gt;...Not to exceed 5 per centum of any appropriation made available to the National Aeronautics and Space Administration...&lt;/content&gt;
+&lt;/appropriations&gt;
+&lt;/appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;title&gt;
+   &lt;appropriations&gt;
+    &lt;appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>93140-93171</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>84 Stat. 1770</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>84</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>91 Session 2</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Two distinct section tags both labeled Sec. 114 in TITLE I of the same pLaw</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>The second Sec. 114 (Congregate housing for the displaced, elderly, and handicapped) should be Sec. 115 — the numbering then continues at Sec. 116, Sec. 117, etc., confirming a missing Sec. 115 in the source XML.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;use of certain housing facilities under section 221 and section 236 for classroom purposes&lt;/heading&gt;
+&lt;num value="114"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 114. &lt;/num&gt;...
+&lt;/section&gt;
+&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;congregate housing for the displaced, elderly, and handicapped&lt;/heading&gt;
+&lt;num value="114"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 114. &lt;/num&gt;...
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;title&gt;
+   &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>108466-108505</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>84 Stat. 1872</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>84</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>91 Session 2</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Bare introductory section element with no num collides with Section 1 in the same pLaw</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Remove the leading bare &lt;section class="inline"&gt;&lt;content&gt;That—&lt;/content&gt;&lt;/section&gt; wrapper — it is the enacting clause continuation and should not be its own &lt;section&gt;. With it removed, Section 1 (which carries num value="1") becomes the only Sec. 1 in the pLaw.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>&lt;section class="inline"&gt;
+&lt;content class="inline"&gt;That—&lt;/content&gt;
+&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;&lt;content class="inline"&gt;Section 204(b) of the Central Intelligence Agency Retirement Act of 1064 for Certain Employees, as amended (78 Stat. 1043; 50 U.S.C. 403 note), is amended by striking subsection (3) and inserting the following in lieu thereof:...&lt;/content&gt;
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>112842-112853</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>84 Stat. 2048</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>84</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>91 Session 2</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Sec. 7 is split into two separate section tags (one carrying subsection (a), the other carrying subsection (b)) instead of one section containing both subsections</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Merge the two consecutive &lt;section&gt;&lt;num value="7"&gt;Sec. 7&lt;/num&gt;...&lt;/section&gt; blocks into a single &lt;section&gt;&lt;num value="7"&gt;Sec. 7&lt;/num&gt; with subsections (a) and (b) inside it, matching the structure of the surrounding sections (Sec. 6, Sec. 8, Sec. 9).</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>&lt;section class="firstIndent1 fontsize10"&gt;&lt;num value="7"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 7&lt;/num&gt;&lt;subsection class="inline"&gt;&lt;num value="a"&gt;(a). &lt;/num&gt;...Subsections (a) and (b) of section 14 of the Food Stamp Act of 1964...
+&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;&lt;num value="7"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 7&lt;/num&gt;&lt;subsection class="inline"&gt;&lt;num value="b"&gt;(b). &lt;/num&gt;&lt;content&gt;Section 14 of the Food Stamp Act of 1964, as amended, is amended by adding the following new subsection:...
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>120966-120980</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>85 Stat. 40</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>85</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>92 Session 1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Two appropriations blocks with the same case-folded heading text collapse to the same UniqueKey</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>The two appropriations blocks under LEGISLATIVE BRANCH with the heading "Contingent Expenses of the Senate" (one Title Case at line 5001, one lowercase at line 5065) should be disambiguated either by nesting the lowercase one inside the preceding "Joint Items" intermediate appropriations block (its closing tag at line 5064 appears to close Joint Items prematurely) or by giving each a distinct heading text. The extractor's heading-derived UniqueKey position collapses both into the same value because the headings are identical after case-folding.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>&lt;appropriations level="intermediate"&gt;&lt;heading&gt;Contingent Expenses of the Senate&lt;/heading&gt;
+&lt;content class="firstIndent1 fontsize10"&gt;
+&lt;list&gt;
+&lt;listItem&gt;&lt;listContent class="firstIndent1 fontsize10 depth0"&gt;“Senate policy committees”, $40,890;&lt;/listContent&gt;&lt;/listItem&gt;
+&lt;listItem&gt;&lt;listContent class="firstIndent1 fontsize10 depth0"&gt;“Automobiles and maintenance”, $3,980;...&lt;/listContent&gt;&lt;/listItem&gt;
+...
+&lt;/list&gt;
+&lt;/content&gt;
+&lt;/appropriations&gt;
+...
+&lt;appropriations level="intermediate"&gt;&lt;heading&gt;Joint Items&lt;/heading&gt;
+&lt;content class="firstIndent1 fontsize10"&gt;
+&lt;list&gt;
+&lt;listItem&gt;&lt;listContent class="firstIndent1 fontsize10 depth0"&gt;“Joint Committee on Reduction of Federal Expenditures”, $5,440, to remain available until expended;&lt;/listContent&gt;&lt;/listItem&gt;
+&lt;/list&gt;
+&lt;/content&gt;
+&lt;/appropriations&gt;
+&lt;appropriations level="small"&gt;&lt;heading&gt;contingent expenses of the senate&lt;/heading&gt;
+&lt;content class="firstIndent1 fontsize10"&gt;
+&lt;list&gt;
+&lt;listItem&gt;&lt;listContent class="firstIndent1 fontsize10 depth0"&gt;“Joint Economic Committee”, $43,195;&lt;/listContent&gt;&lt;/listItem&gt;
+&lt;listItem&gt;&lt;listContent class="firstIndent1 fontsize10 depth0"&gt;“Joint Committee on Atomic Energy”, $27,285;&lt;/listContent&gt;&lt;/listItem&gt;
+&lt;listItem&gt;&lt;listContent class="firstIndent1 fontsize10 depth0"&gt;“Joint Committee on Printing”, $19,405;&lt;/listContent&gt;&lt;/listItem&gt;
+&lt;/list&gt;
+&lt;/content&gt;
+&lt;/appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;appropriations&gt;
+   &lt;appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>5001-5073</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>85 Stat. 682</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>85</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>92 Session 1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Unnumbered introductory section collides with the law's numbered Sec. 1 in the UniqueKey</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>The introductory section at line 36523 (a "section" element with no "num" child, containing the "That the following sums are appropriated" enacting text) collapses to the same UniqueKey SectionNumber position as the later "Sec. 1." general-provisions section at line 36575. The unnumbered enacting-clause section should either be excluded from the section row inventory or be assigned a distinct SectionNumber position so it does not collide with the numbered Sec. 1.</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>&lt;section class="inline"&gt;
+&lt;content class="inline"&gt;That the following sums are appropriated, out of any money in the Treasury not otherwise appropriated, for the District of Columbia for the fiscal year ending June 30, 1972, and for other purposes, namely:&lt;/content&gt;
+&lt;/section&gt;
+...
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 1. &lt;/num&gt;&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;Vouchers.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;content class="inline"&gt;Except as otherwise provided herein, all vouchers covering expenditures of appropriations contained in this Act shall be audited before payment by the designated certifying official and the vouchers as approved shall be paid by checks issued by the designated disbursing official without countersignature.&lt;/content&gt;
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>36523-36580</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>86 Stat. 688</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>86</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>92 Session 2</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Law number reported as 4424 between Public Law 92-423 and Public Law 92-425</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Should be Public Law 92-424 — the same pLaw's dc:title, docNumber, and preface docNumber all read 92-424; only the citableAs has the extra digit.</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>&lt;dc:title&gt;Public Law 92–424: To provide for the continuation of programs authorized under the Economic Opportunity Act of 1964, and for other purposes.&lt;/dc:title&gt;
+&lt;dc:type&gt;Public Law&lt;/dc:type&gt;
+&lt;docNumber&gt;424&lt;/docNumber&gt;
+&lt;citableAs&gt;Public Law 92–4424&lt;/citableAs&gt;
+&lt;citableAs&gt;86 Stat. 688&lt;/citableAs&gt;</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;meta&gt;
+  &lt;docNumber&gt;
+   &lt;citableAs&gt;</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>38864-39653</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>86 Stat. 706</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>86</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>92 Session 2</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Reviewed: gap — no correction needed</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Legitimate placement — the apparent gap between 4424 and 425 is an artifact of the OCR error in the preceding pLaw's citableAs (4424 should read 424). Once 92-4424 is corrected to 92-424, this pLaw's numbering 92-425 is correctly the next in sequence.</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>&lt;dc:title&gt;Public Law 92–425: To amend chapter 73 of title 10, United States Code, to establish a Survivor Benefit Plan, and tor other purposes.&lt;/dc:title&gt;
+&lt;dc:type&gt;Public Law&lt;/dc:type&gt;
+&lt;docNumber&gt;425&lt;/docNumber&gt;
+&lt;citableAs&gt;Public Law 92–425&lt;/citableAs&gt;
+&lt;citableAs&gt;86 Stat. 706&lt;/citableAs&gt;
+&lt;approvedDate&gt;1972-09-21&lt;/approvedDate&gt;</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;meta&gt;
+  &lt;docNumber&gt;
+   &lt;citableAs&gt;</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>39659-40050</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>86 Stat. 451</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>86</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>92 Session 2</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Duplicate section UniqueKey collision between the enacting clause and the explicit Section 1</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>The enacting &lt;section&gt; (no &lt;num&gt;) and the later &lt;section&gt;&lt;num value="1"&gt;Section 1.&lt;/num&gt; both map to UniqueKey position 001 and need to be distinguished — either tag the unnumbered enacting section with a distinct ordinal namespace or start null-section ordinals after the highest explicit section number in the pLaw.</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>&lt;section class="inline"&gt;
+&lt;content class="inline"&gt;That the following &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;District of Columbia Appropriation Act, 1973.&lt;/p&gt;&lt;/sidenote&gt;sums are appropriated, out of any money in the Treasury not otherwise appropriated, for the District of Columbia for the fiscal year ending J line 30, 1973, and for other purposes, namely:&lt;/content&gt;
+&lt;/section&gt;
+...
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;Vouchers.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;content&gt;Except as otherwise provided herein, all vouchers covering expenditures of appropriations contained in this Act shall be audited before payment by the designated certifying official and the vouchers as approved shall be paid by checks issued by the designated disbursing official.&lt;/content&gt;
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>28444-28642</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>86 Stat. 471</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>86</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>92 Session 2</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Two sibling level blocks under Title IV each contain their own Sec. 1 — the level heading is not captured so both Sec. 1 rows share the same UniqueKey</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Carry the &lt;level&gt;&lt;heading&gt; text (General Provisions—General Services Administration vs General Provisions—Civil Defense) into a DivisionHeading slot so that the two Sec. 1 sections under Title IV produce distinct UniqueKey paths.</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>&lt;level&gt;
+&lt;heading class="smallCaps centered"&gt;General Provisions—General Services Administration&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 1 &lt;/num&gt;
+&lt;content class="inline"&gt;The appropriate appropriation or fund available to the General Services Administration shall be credited with...&lt;/content&gt;
+&lt;/section&gt;
+...
+&lt;/level&gt;
+...
+&lt;level&gt;
+&lt;heading class="smallCaps centered"&gt;General Provisions—Civil Defense&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 1. &lt;/num&gt;
+&lt;content class="inline"&gt;Appropriations contained in this Act for carrying out civil defense activities shall not be available in excess of the limitations on appropriations contained in section 408 of the Federal Civil Defense Act, as amended (50 U.S.C. App. 2260).&lt;/content&gt;
+&lt;/section&gt;
+...
+&lt;/level&gt;</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;title&gt;
+   &lt;level&gt;
+    &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>29439-30098</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>86 Stat. 471</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>86</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>92 Session 2</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Two sibling level blocks under Title IV each contain their own Sec. 2 — the level heading is not captured so both Sec. 2 rows share the same UniqueKey</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Carry the &lt;level&gt;&lt;heading&gt; text (General Provisions—General Services Administration vs General Provisions—Civil Defense) into a DivisionHeading slot so that the two Sec. 2 sections under Title IV produce distinct UniqueKey paths.</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>&lt;level&gt;
+&lt;heading class="smallCaps centered"&gt;General Provisions—General Services Administration&lt;/heading&gt;
+...
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 2. &lt;/num&gt;
+&lt;content class="inline"&gt;Appropriations to the General Services Administration under the heading “Construction, Public Buildings Projects” shall be available, subject to the provisions of the Public Buildings Act of 1959 for (1) acquisition of buildings and sites thereof by purchase, condemnation, or otherwise...&lt;/content&gt;
+&lt;/section&gt;
+&lt;/level&gt;
+...
+&lt;level&gt;
+&lt;heading class="smallCaps centered"&gt;General Provisions—Civil Defense&lt;/heading&gt;
+...
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 2. &lt;/num&gt;
+&lt;content class="inline"&gt;No part of any appropriation in this Act shall be available for the construction of warehouses or for the lease of warehouse space in any building which is to be constructed specifically for civil defense activities.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/level&gt;</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;title&gt;
+   &lt;level&gt;
+    &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>29439-30098</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>86 Stat. 722</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>86</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>92 Session 2</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Reviewed: duplicate UniqueKey — covered by an existing approved correction</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Two adjacent sections with no &lt;num&gt; (one enacting clause introducing the amendment, one whose body is wrapped in &lt;quotedContent&gt;) collapse to UniqueKey position 001. This is the same shape as approved correction #2 (PL 87-292 / PL 87-356); the sequential intra-law ordinal logic will assign 1 and 2 respectively and resolve the collision.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;content&gt;That section 500 of title 18, United States Code, as amended by section 6(j)(5) of the Postal Reorganization Act, Public Law 91–375, is further amended to read as follows:&lt;/content&gt;
+&lt;/section&gt;
+&lt;section&gt;
+&lt;quotedContent&gt;
+“§ 500. Money orders
+“Whoever, with intent to defraud, falsely makes, forges, counterfeits, engraves, or prints any order in imitation of or purporting to be a blank money order or a money order issued by or under the direction of the Post Office Department or Postal Service; or
+...
+&lt;/quotedContent&gt;
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>40546-40612</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>87 Stat. 306</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>87</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>93 Session 1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Opening unnumbered "That..." section collides with a later numbered Sec. 1. in the same Act</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>The opening &lt;section class="inline"&gt; carrying the enacting "That the following sums are appropriated..." paragraph has no &lt;num&gt; child, so the extractor places it in the same SectionNumber slot as the General Provisions "Sec. 1." later in the Act. The opening preamble section should be tracked in a distinct slot (or merged with the enacting formula) so that its UniqueKey does not collide with Sec. 1.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>&lt;section class="inline"&gt;
+&lt;content class="inline"&gt;That the following sums are appropriated, out of any money in the Treasury not otherwise appropriated, for the District of Columbia for the fiscal year ending June 30, 1974, and for other purposes, namely:&lt;/content&gt;
+&lt;/section&gt;
+...
+&lt;level&gt;
+&lt;heading class="centered"&gt;GENERAL PROVISIONS&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num class="smallCaps" value="1"&gt;Sec. 1. &lt;/num&gt;
+&lt;content class="inline"&gt;Except as otherwise provided herein, all vouchers covering expenditures of appropriations contained in this Act shall be audited before payment by the designated certifying official and the vouchers as approved shall be paid by checks issued by the designated disbursing official.&lt;/content&gt;
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>17431-17481</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>87 Stat. 455</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>87</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>93 Session 1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Two sections both labeled "Sec. 3." in the same Act (the second one should be Sec. 5.)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>The fifth section of this Act is mislabeled in the source XML as "Sec. 3." (&lt;num value="3"&gt;), creating a duplicate of the real Sec. 3. The element should read "Sec. 5." (&lt;num value="5"&gt;) so the section sequence (1 - opening "That ...", 2, 3, 4, 5) is consistent with the printed Statutes.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 3. &lt;/num&gt;&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;Manufacture and storage.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;content class="inline"&gt;Until the Secretary of the Treasury determines that the mints of the United States are adequate for the production of ample supplies of coins and medals, any facility of the Bureau of the Mint may be used for the manufacture and storage of medals and coins.&lt;/content&gt;
+&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="4"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 4. &lt;/num&gt;&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;Silver-clad coins, limitations.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;content class="inline"&gt;Notwithstanding any other provision of law with respect to the design of coins, the Secretary shall mint prior to July 4, 1975, for issuance on and after such date, 45 million silver-clad alloy coins...&lt;/content&gt;
+&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 3. &lt;/num&gt;&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;Numismatic items, distribution.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;content class="inline"&gt;In connection with the operations of the Bureau of the Mint, the Secretary of the Treasury is authorized to manufacture and distribute numismatic items. Proceeds from the sale of numismatic items shall be reimbursed to the current appropriation for the cost of manufacturing and handling of such items.&lt;/content&gt;
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>23741-23752</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>87 Stat. 471</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>87</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>93 Session 1</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Two sibling &lt;appropriations&gt; elements under SCIENCE AND EDUCATION PROGRAMS share the heading "animal and plant health inspection service" — the second one is mislabeled and should read "cooperative state research service"</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>The second &lt;heading&gt;animal and plant health inspection service&lt;/heading&gt; at line 24714 is mislabeled in the source XML. Its content is about payments to agricultural experiment stations, the Hatch Act, cooperative forestry research, and the Cooperative State Research Service — the heading should read "cooperative state research service". The heading-derived UniqueKey collision is otherwise handled by the existing sibling-heading ordinal disambiguation (active correction #5), so this row needs a source-XML heading fix at GPO rather than an extractor change.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>&lt;appropriations level="small"&gt;&lt;heading&gt;animal and plant health inspection service&lt;/heading&gt;
+&lt;content&gt;For expenses, not otherwise provided for, including those pursuant to the Act of February 28, 1947, as amended (21 U.S.C. 114b-c) necessary to prevent, control, and eradicate pests and plant and animal diseases; to carry out inspection, quarantine and regulatory activities; to carry on services related to consumer protection: and to protect the environment, as authorized by law. $285,925,000 ...&lt;/content&gt;
+&lt;/appropriations&gt;
+&lt;appropriations level="small"&gt;&lt;heading&gt;animal and plant health inspection service&lt;/heading&gt;
+&lt;content&gt;For payments to agricultural experiment stations, for grants for cooperative forestry and other research, for facilities, and for other expenses, including $70,104,000 to carry into effect the provisions of the Hatch Act, approved March 2, 1887, as amended by the Act approved August 11, 1955 (7. U.S.C. 361a-361i), and further amended by Public Law 92-318 approved June 23, 1972, including administration by the United States Department of Agriculture, and penalty mail costs of agricultural experiment stations under section 6 of the Hatch Act of 1887, as amended; ... $89,880,000.&lt;/content&gt;
+&lt;/appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;title&gt;
+   &lt;appropriations&gt;
+    &lt;appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>24711-24716</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>88 Stat. 96</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>88</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 30 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content&gt;This Act may be cited as the “Federal Energy Administration&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t15/s761"&gt;15 USC 761 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; Act of 1974”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>6815-6821</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>88 Stat. 125</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>88</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 2 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content class="inline"&gt;This title may be cited as the “Comprehensive Alcohol&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;Comprehensive Alcohol Abuse and Alcoholism Prevention, Treatment, and Rehabilitation Act Amendments of 1974.&lt;/p&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s4541"&gt;42 USC 4541 note&lt;/ref&gt;.&lt;/p&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s4551"&gt;42 USC 4551 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; Abuse and Alcoholism Prevention, Treatment, and Rehabilitation Act Amendments of 1974”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>8568-8574</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>88 Stat. 143</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>88</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 2 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;findings and declarations&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;The Congress hereby finds and declares that—&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s5121"&gt;42 USC 5121&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;&lt;/chapeau&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content class="inline"&gt;because disasters often cause loss of life, human suffering, loss of income, and property loss and damage; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content class="inline"&gt;because disasters often disrupt the normal functioning of governments and communities, and adversely affect individuals and families with great severity;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;continuation class="inline"&gt;special measures, designed to assist the efforts of the affected States in expediting the rendering of aid, assistance, and emergency services, and the reconstruction and rehabilitation of devastated areas, are necessary.&lt;/continuation&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;It is the intent of the Congress, by this Act, to provide an orderly and continuing means of assistance by the Federal Government to State and local governments in carrying out their responsibilities to alleviate the suffering and damage which result from such disasters by—&lt;/chapeau&gt;
+&lt;page identifier="/us/stat/88/144"&gt;88 &lt;inline class="smallCaps"&gt;Stat&lt;/inline&gt;. 144&lt;/page&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content class="inline"&gt;revising and broadening the scope of existing disaster relief programs;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging the development of comprehensive disaster preparedness and assistance plans, programs, capabilities, and organizations by the States and by local governments;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;(3) &lt;/num&gt;
+&lt;content class="inline"&gt;achieving greater coordination and responsiveness of disaster preparedness and relief programs;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="4"&gt;(4) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging individuals, States, and local governments to protect themselves by obtaining insurance coverage to supplement or replace governmental assistance;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="5"&gt;(5) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging hazard mitigation measures to reduce losses from disasters, including development of land use and construction regulations;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="6"&gt;(6) &lt;/num&gt;
+&lt;content class="inline"&gt;providing Federal assistance programs for both public and private losses sustained in disasters; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="7"&gt;(7) &lt;/num&gt;
+&lt;content class="inline"&gt;providing a long-range economic recovery program for major disaster areas.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;/subsection&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>9784-9835</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>88 Stat. 143</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>88</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 18 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;findings and declarations&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;The Congress hereby finds and declares that—&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s5121"&gt;42 USC 5121&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;&lt;/chapeau&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content class="inline"&gt;because disasters often cause loss of life, human suffering, loss of income, and property loss and damage; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content class="inline"&gt;because disasters often disrupt the normal functioning of governments and communities, and adversely affect individuals and families with great severity;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;continuation class="inline"&gt;special measures, designed to assist the efforts of the affected States in expediting the rendering of aid, assistance, and emergency services, and the reconstruction and rehabilitation of devastated areas, are necessary.&lt;/continuation&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;It is the intent of the Congress, by this Act, to provide an orderly and continuing means of assistance by the Federal Government to State and local governments in carrying out their responsibilities to alleviate the suffering and damage which result from such disasters by—&lt;/chapeau&gt;
+&lt;page identifier="/us/stat/88/144"&gt;88 &lt;inline class="smallCaps"&gt;Stat&lt;/inline&gt;. 144&lt;/page&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content class="inline"&gt;revising and broadening the scope of existing disaster relief programs;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging the development of comprehensive disaster preparedness and assistance plans, programs, capabilities, and organizations by the States and by local governments;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;(3) &lt;/num&gt;
+&lt;content class="inline"&gt;achieving greater coordination and responsiveness of disaster preparedness and relief programs;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="4"&gt;(4) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging individuals, States, and local governments to protect themselves by obtaining insurance coverage to supplement or replace governmental assistance;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="5"&gt;(5) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging hazard mitigation measures to reduce losses from disasters, including development of land use and construction regulations;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="6"&gt;(6) &lt;/num&gt;
+&lt;content class="inline"&gt;providing Federal assistance programs for both public and private losses sustained in disasters; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="7"&gt;(7) &lt;/num&gt;
+&lt;content class="inline"&gt;providing a long-range economic recovery program for major disaster areas.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;/subsection&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>9784-9835</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>88 Stat. 143</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>88</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 19 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;findings and declarations&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;The Congress hereby finds and declares that—&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s5121"&gt;42 USC 5121&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;&lt;/chapeau&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content class="inline"&gt;because disasters often cause loss of life, human suffering, loss of income, and property loss and damage; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content class="inline"&gt;because disasters often disrupt the normal functioning of governments and communities, and adversely affect individuals and families with great severity;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;continuation class="inline"&gt;special measures, designed to assist the efforts of the affected States in expediting the rendering of aid, assistance, and emergency services, and the reconstruction and rehabilitation of devastated areas, are necessary.&lt;/continuation&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;It is the intent of the Congress, by this Act, to provide an orderly and continuing means of assistance by the Federal Government to State and local governments in carrying out their responsibilities to alleviate the suffering and damage which result from such disasters by—&lt;/chapeau&gt;
+&lt;page identifier="/us/stat/88/144"&gt;88 &lt;inline class="smallCaps"&gt;Stat&lt;/inline&gt;. 144&lt;/page&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content class="inline"&gt;revising and broadening the scope of existing disaster relief programs;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging the development of comprehensive disaster preparedness and assistance plans, programs, capabilities, and organizations by the States and by local governments;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;(3) &lt;/num&gt;
+&lt;content class="inline"&gt;achieving greater coordination and responsiveness of disaster preparedness and relief programs;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="4"&gt;(4) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging individuals, States, and local governments to protect themselves by obtaining insurance coverage to supplement or replace governmental assistance;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="5"&gt;(5) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging hazard mitigation measures to reduce losses from disasters, including development of land use and construction regulations;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="6"&gt;(6) &lt;/num&gt;
+&lt;content class="inline"&gt;providing Federal assistance programs for both public and private losses sustained in disasters; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="7"&gt;(7) &lt;/num&gt;
+&lt;content class="inline"&gt;providing a long-range economic recovery program for major disaster areas.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;/subsection&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>9784-9835</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>88 Stat. 143</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>88</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 6 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;findings and declarations&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;The Congress hereby finds and declares that—&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s5121"&gt;42 USC 5121&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;&lt;/chapeau&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content class="inline"&gt;because disasters often cause loss of life, human suffering, loss of income, and property loss and damage; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content class="inline"&gt;because disasters often disrupt the normal functioning of governments and communities, and adversely affect individuals and families with great severity;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;continuation class="inline"&gt;special measures, designed to assist the efforts of the affected States in expediting the rendering of aid, assistance, and emergency services, and the reconstruction and rehabilitation of devastated areas, are necessary.&lt;/continuation&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;It is the intent of the Congress, by this Act, to provide an orderly and continuing means of assistance by the Federal Government to State and local governments in carrying out their responsibilities to alleviate the suffering and damage which result from such disasters by—&lt;/chapeau&gt;
+&lt;page identifier="/us/stat/88/144"&gt;88 &lt;inline class="smallCaps"&gt;Stat&lt;/inline&gt;. 144&lt;/page&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content class="inline"&gt;revising and broadening the scope of existing disaster relief programs;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging the development of comprehensive disaster preparedness and assistance plans, programs, capabilities, and organizations by the States and by local governments;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;(3) &lt;/num&gt;
+&lt;content class="inline"&gt;achieving greater coordination and responsiveness of disaster preparedness and relief programs;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="4"&gt;(4) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging individuals, States, and local governments to protect themselves by obtaining insurance coverage to supplement or replace governmental assistance;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="5"&gt;(5) &lt;/num&gt;
+&lt;content class="inline"&gt;encouraging hazard mitigation measures to reduce losses from disasters, including development of land use and construction regulations;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="6"&gt;(6) &lt;/num&gt;
+&lt;content class="inline"&gt;providing Federal assistance programs for both public and private losses sustained in disasters; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="7"&gt;(7) &lt;/num&gt;
+&lt;content class="inline"&gt;providing a long-range economic recovery program for major disaster areas.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;/subsection&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>9784-9835</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>88 Stat. 237</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>88</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 4 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;authorization of appropriations &lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content class="inline"&gt;Section 2(a) (1) of the Department of State Appropriations Authorization Act of 1973 (87 Stat. 451), providing authorization of appropriations for the Administration of Foreign Affairs, is amended by striking out “&lt;quotedText&gt;$282,565,000&lt;/quotedText&gt;” and inserting in lieu thereof “&lt;quotedText&gt;$304,568,000&lt;/quotedText&gt;”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>16522-16528</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>88 Stat. 286</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>88</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 7 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;commodity distribution program&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 2 &lt;/num&gt;
+&lt;content class="inline"&gt;The National School Lunch Act (42 U.S.C. 1751 et seq.) is amended by redesignating section 14 as section 15 and by inserting&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s1763"&gt;42 USC 1763&lt;/ref&gt;.&lt;/p&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s1762"&gt;42 USC 1762&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; immediately after section IBA the following new section:
+&lt;quotedContent&gt;
+&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;“commodity distribution program&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="14"&gt;“&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 14. &lt;/num&gt;
+&lt;chapeau class="inline"&gt;Notwithstanding any other provision of law, the Secretary, &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s1762a"&gt;42 USC 1762a&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; during the period beginning July 1, 1974, and ending June 30, 1975, shall—&lt;/chapeau&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;“(1) &lt;/num&gt;
+&lt;content class="inline"&gt;use funds available to carry out the provisions of section 32 of the Act of August 24, 1935 (7 U.S.C. 612c) which are not expended or needed to carry out such provisions, to purchase (without regard to the provisions of existing law governing the expenditure of public funds) agricultural commodities and their products of the types customarily purchased under such section, for donation to maintain the annually programmed level of assistance for programs carried on under this Act, the Child Nutrition Act of 1966, and title V I I of the Older Americans Act&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s1771"&gt;42 USC 1771 note&lt;/ref&gt;.&lt;/p&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s3045"&gt;42 USC 3045&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; of 1965; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;“(2) &lt;/num&gt;
+&lt;content class="inline"&gt;if stocks of the Commodity Credit Corporation are not available, use the funds of such Corporation to purchase agricultural commodities and their products of the types customarily available under section 416 of the Agricultural Act of 1949 (7 U.S.C. 1431), for such donation.”.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+&lt;/quotedContent&gt;
+&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>19164-19188</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>88 Stat. 297</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>88</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 3 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short titles; table of contents&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Short Titles&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “Congressional Budget and Impoundment Control Act of 1974”. Titles I through IX may be cited as the “Congressional Budget Act of 1974”, and title X may be cited as the “Impoundment Control Act of 1974”.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Table of Contents&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content&gt;
+&lt;toc&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 1.&lt;/designator&gt; &lt;label&gt;Short titles; table of contents.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 2.&lt;/designator&gt; &lt;label&gt;Declaration of purposes.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 3.&lt;/designator&gt; &lt;label&gt;Definitions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE I—&lt;/designator&gt; &lt;label class="centered"&gt;ESTABLISHMENT OF HOUSE AND SENATE BUDGET COMMITTEES&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 101.&lt;/designator&gt; &lt;label&gt;Budget Committee of the House of Representatives.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 102.&lt;/designator&gt; &lt;label&gt;Budget Committee of the Senate.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE II—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET OFFICE&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 201. &lt;/designator&gt;&lt;label&gt;Establishment of Office.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 202.&lt;/designator&gt; &lt;label&gt;Duties and functions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 203.&lt;/designator&gt; &lt;label&gt;Public access to budget data.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE III—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET PROCESS&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 300.&lt;/designator&gt; &lt;label&gt;Timetable.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 301.&lt;/designator&gt; &lt;label&gt;Adoption of first concurrent resolution.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 302.&lt;/designator&gt; &lt;label&gt;Matters to be included in joint statement of managers; reports by committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 303.&lt;/designator&gt; &lt;label&gt;First concurrent resolution on the budget must be adopted before legislation providing new budget authority, new spending authority, or changes in revenues or public debt limit is considered.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 304.&lt;/designator&gt; &lt;label&gt;Permissible revisions of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 305.&lt;/designator&gt; &lt;label&gt;Provisions relating to the consideration of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 306.&lt;/designator&gt; &lt;label&gt;Legislation dealing with congressional budget must be handled by budget committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 307.&lt;/designator&gt; &lt;label&gt;House committee action on all appropriation bills to be completed before first appropriation bill is reported.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 308.&lt;/designator&gt; &lt;label&gt;Reports, summaries, and projections of congressional budget actions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 309.&lt;/designator&gt; &lt;label&gt;Completion of act
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>20300-20411</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>88 Stat. 297</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>88</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 2 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short titles; table of contents&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Short Titles&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “Congressional Budget and Impoundment Control Act of 1974”. Titles I through IX may be cited as the “Congressional Budget Act of 1974”, and title X may be cited as the “Impoundment Control Act of 1974”.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Table of Contents&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content&gt;
+&lt;toc&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 1.&lt;/designator&gt; &lt;label&gt;Short titles; table of contents.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 2.&lt;/designator&gt; &lt;label&gt;Declaration of purposes.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 3.&lt;/designator&gt; &lt;label&gt;Definitions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE I—&lt;/designator&gt; &lt;label class="centered"&gt;ESTABLISHMENT OF HOUSE AND SENATE BUDGET COMMITTEES&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 101.&lt;/designator&gt; &lt;label&gt;Budget Committee of the House of Representatives.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 102.&lt;/designator&gt; &lt;label&gt;Budget Committee of the Senate.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE II—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET OFFICE&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 201. &lt;/designator&gt;&lt;label&gt;Establishment of Office.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 202.&lt;/designator&gt; &lt;label&gt;Duties and functions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 203.&lt;/designator&gt; &lt;label&gt;Public access to budget data.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE III—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET PROCESS&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 300.&lt;/designator&gt; &lt;label&gt;Timetable.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 301.&lt;/designator&gt; &lt;label&gt;Adoption of first concurrent resolution.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 302.&lt;/designator&gt; &lt;label&gt;Matters to be included in joint statement of managers; reports by committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 303.&lt;/designator&gt; &lt;label&gt;First concurrent resolution on the budget must be adopted before legislation providing new budget authority, new spending authority, or changes in revenues or public debt limit is considered.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 304.&lt;/designator&gt; &lt;label&gt;Permissible revisions of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 305.&lt;/designator&gt; &lt;label&gt;Provisions relating to the consideration of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 306.&lt;/designator&gt; &lt;label&gt;Legislation dealing with congressional budget must be handled by budget committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 307.&lt;/designator&gt; &lt;label&gt;House committee action on all appropriation bills to be completed before first appropriation bill is reported.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 308.&lt;/designator&gt; &lt;label&gt;Reports, summaries, and projections of congressional budget actions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 309.&lt;/designator&gt; &lt;label&gt;Completion of act
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>20300-20411</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>88 Stat. 297</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>88</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 12 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short titles; table of contents&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Short Titles&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “Congressional Budget and Impoundment Control Act of 1974”. Titles I through IX may be cited as the “Congressional Budget Act of 1974”, and title X may be cited as the “Impoundment Control Act of 1974”.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Table of Contents&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content&gt;
+&lt;toc&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 1.&lt;/designator&gt; &lt;label&gt;Short titles; table of contents.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 2.&lt;/designator&gt; &lt;label&gt;Declaration of purposes.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 3.&lt;/designator&gt; &lt;label&gt;Definitions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE I—&lt;/designator&gt; &lt;label class="centered"&gt;ESTABLISHMENT OF HOUSE AND SENATE BUDGET COMMITTEES&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 101.&lt;/designator&gt; &lt;label&gt;Budget Committee of the House of Representatives.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 102.&lt;/designator&gt; &lt;label&gt;Budget Committee of the Senate.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE II—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET OFFICE&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 201. &lt;/designator&gt;&lt;label&gt;Establishment of Office.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 202.&lt;/designator&gt; &lt;label&gt;Duties and functions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 203.&lt;/designator&gt; &lt;label&gt;Public access to budget data.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE III—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET PROCESS&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 300.&lt;/designator&gt; &lt;label&gt;Timetable.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 301.&lt;/designator&gt; &lt;label&gt;Adoption of first concurrent resolution.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 302.&lt;/designator&gt; &lt;label&gt;Matters to be included in joint statement of managers; reports by committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 303.&lt;/designator&gt; &lt;label&gt;First concurrent resolution on the budget must be adopted before legislation providing new budget authority, new spending authority, or changes in revenues or public debt limit is considered.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 304.&lt;/designator&gt; &lt;label&gt;Permissible revisions of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 305.&lt;/designator&gt; &lt;label&gt;Provisions relating to the consideration of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 306.&lt;/designator&gt; &lt;label&gt;Legislation dealing with congressional budget must be handled by budget committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 307.&lt;/designator&gt; &lt;label&gt;House committee action on all appropriation bills to be completed before first appropriation bill is reported.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 308.&lt;/designator&gt; &lt;label&gt;Reports, summaries, and projections of congressional budget actions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 309.&lt;/designator&gt; &lt;label&gt;Completion of act
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>20300-20411</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>88 Stat. 297</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>88</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 4 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short titles; table of contents&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Short Titles&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “Congressional Budget and Impoundment Control Act of 1974”. Titles I through IX may be cited as the “Congressional Budget Act of 1974”, and title X may be cited as the “Impoundment Control Act of 1974”.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Table of Contents&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content&gt;
+&lt;toc&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 1.&lt;/designator&gt; &lt;label&gt;Short titles; table of contents.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 2.&lt;/designator&gt; &lt;label&gt;Declaration of purposes.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 3.&lt;/designator&gt; &lt;label&gt;Definitions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE I—&lt;/designator&gt; &lt;label class="centered"&gt;ESTABLISHMENT OF HOUSE AND SENATE BUDGET COMMITTEES&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 101.&lt;/designator&gt; &lt;label&gt;Budget Committee of the House of Representatives.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 102.&lt;/designator&gt; &lt;label&gt;Budget Committee of the Senate.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE II—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET OFFICE&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 201. &lt;/designator&gt;&lt;label&gt;Establishment of Office.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 202.&lt;/designator&gt; &lt;label&gt;Duties and functions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 203.&lt;/designator&gt; &lt;label&gt;Public access to budget data.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE III—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET PROCESS&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 300.&lt;/designator&gt; &lt;label&gt;Timetable.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 301.&lt;/designator&gt; &lt;label&gt;Adoption of first concurrent resolution.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 302.&lt;/designator&gt; &lt;label&gt;Matters to be included in joint statement of managers; reports by committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 303.&lt;/designator&gt; &lt;label&gt;First concurrent resolution on the budget must be adopted before legislation providing new budget authority, new spending authority, or changes in revenues or public debt limit is considered.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 304.&lt;/designator&gt; &lt;label&gt;Permissible revisions of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 305.&lt;/designator&gt; &lt;label&gt;Provisions relating to the consideration of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 306.&lt;/designator&gt; &lt;label&gt;Legislation dealing with congressional budget must be handled by budget committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 307.&lt;/designator&gt; &lt;label&gt;House committee action on all appropriation bills to be completed before first appropriation bill is reported.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 308.&lt;/designator&gt; &lt;label&gt;Reports, summaries, and projections of congressional budget actions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 309.&lt;/designator&gt; &lt;label&gt;Completion of act
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>20300-20411</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>88 Stat. 297</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>88</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 6 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short titles; table of contents&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Short Titles&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “Congressional Budget and Impoundment Control Act of 1974”. Titles I through IX may be cited as the “Congressional Budget Act of 1974”, and title X may be cited as the “Impoundment Control Act of 1974”.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Table of Contents&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content&gt;
+&lt;toc&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 1.&lt;/designator&gt; &lt;label&gt;Short titles; table of contents.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 2.&lt;/designator&gt; &lt;label&gt;Declaration of purposes.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 3.&lt;/designator&gt; &lt;label&gt;Definitions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE I—&lt;/designator&gt; &lt;label class="centered"&gt;ESTABLISHMENT OF HOUSE AND SENATE BUDGET COMMITTEES&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 101.&lt;/designator&gt; &lt;label&gt;Budget Committee of the House of Representatives.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 102.&lt;/designator&gt; &lt;label&gt;Budget Committee of the Senate.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE II—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET OFFICE&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 201. &lt;/designator&gt;&lt;label&gt;Establishment of Office.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 202.&lt;/designator&gt; &lt;label&gt;Duties and functions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 203.&lt;/designator&gt; &lt;label&gt;Public access to budget data.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE III—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET PROCESS&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 300.&lt;/designator&gt; &lt;label&gt;Timetable.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 301.&lt;/designator&gt; &lt;label&gt;Adoption of first concurrent resolution.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 302.&lt;/designator&gt; &lt;label&gt;Matters to be included in joint statement of managers; reports by committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 303.&lt;/designator&gt; &lt;label&gt;First concurrent resolution on the budget must be adopted before legislation providing new budget authority, new spending authority, or changes in revenues or public debt limit is considered.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 304.&lt;/designator&gt; &lt;label&gt;Permissible revisions of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 305.&lt;/designator&gt; &lt;label&gt;Provisions relating to the consideration of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 306.&lt;/designator&gt; &lt;label&gt;Legislation dealing with congressional budget must be handled by budget committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 307.&lt;/designator&gt; &lt;label&gt;House committee action on all appropriation bills to be completed before first appropriation bill is reported.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 308.&lt;/designator&gt; &lt;label&gt;Reports, summaries, and projections of congressional budget actions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 309.&lt;/designator&gt; &lt;label&gt;Completion of act
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>20300-20411</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>88 Stat. 297</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>88</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 7 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short titles; table of contents&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Short Titles&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “Congressional Budget and Impoundment Control Act of 1974”. Titles I through IX may be cited as the “Congressional Budget Act of 1974”, and title X may be cited as the “Impoundment Control Act of 1974”.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;heading class="inline"&gt;&lt;inline class="smallCaps"&gt;Table of Contents&lt;/inline&gt;.—&lt;/heading&gt;
+&lt;content&gt;
+&lt;toc&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 1.&lt;/designator&gt; &lt;label&gt;Short titles; table of contents.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 2.&lt;/designator&gt; &lt;label&gt;Declaration of purposes.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 3.&lt;/designator&gt; &lt;label&gt;Definitions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE I—&lt;/designator&gt; &lt;label class="centered"&gt;ESTABLISHMENT OF HOUSE AND SENATE BUDGET COMMITTEES&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 101.&lt;/designator&gt; &lt;label&gt;Budget Committee of the House of Representatives.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 102.&lt;/designator&gt; &lt;label&gt;Budget Committee of the Senate.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE II—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET OFFICE&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 201. &lt;/designator&gt;&lt;label&gt;Establishment of Office.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 202.&lt;/designator&gt; &lt;label&gt;Duties and functions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 203.&lt;/designator&gt; &lt;label&gt;Public access to budget data.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;/toc&gt;
+&lt;toc&gt;
+&lt;referenceItem role="title"&gt;&lt;designator class="centered"&gt;TITLE III—&lt;/designator&gt; &lt;label class="centered"&gt;CONGRESSIONAL BUDGET PROCESS&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 300.&lt;/designator&gt; &lt;label&gt;Timetable.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 301.&lt;/designator&gt; &lt;label&gt;Adoption of first concurrent resolution.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 302.&lt;/designator&gt; &lt;label&gt;Matters to be included in joint statement of managers; reports by committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 303.&lt;/designator&gt; &lt;label&gt;First concurrent resolution on the budget must be adopted before legislation providing new budget authority, new spending authority, or changes in revenues or public debt limit is considered.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 304.&lt;/designator&gt; &lt;label&gt;Permissible revisions of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 305.&lt;/designator&gt; &lt;label&gt;Provisions relating to the consideration of concurrent resolutions on the budget.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 306.&lt;/designator&gt; &lt;label&gt;Legislation dealing with congressional budget must be handled by budget committees.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 307.&lt;/designator&gt; &lt;label&gt;House committee action on all appropriation bills to be completed before first appropriation bill is reported.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 308.&lt;/designator&gt; &lt;label&gt;Reports, summaries, and projections of congressional budget actions.&lt;/label&gt;&lt;/referenceItem&gt;
+&lt;referenceItem role="section"&gt;&lt;designator&gt;Sec. 309.&lt;/designator&gt; &lt;label&gt;Completion of act
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>20300-20411</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>88 Stat. 342</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>88</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 6 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content class="inline"&gt;This title may be cited as the “National Research Service Award Act of 1974”.&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s289l–1"&gt;42 USC 289&lt;i&gt;l&lt;/i&gt;–1 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>22919-22925</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>88 Stat. 373</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>88</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 6 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “National Diabetes Mellitus Research and Education Act”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s289c–2"&gt;42 USC 289c–2 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>25073-25080</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>88 Stat. 378</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>88</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 2 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 2. &lt;/num&gt;
+&lt;content class="inline"&gt;The Economic Opportunity Act of 1964 is amended by adding at the end thereof the following new title: &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s2701"&gt;42 USC 2701 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;quotedContent&gt;
+&lt;title&gt;
+&lt;num value="X"&gt;“TITLE X—&lt;/num&gt;
+&lt;heading class="inline"&gt;LEGAL SERVICES CORPORATION ACT&lt;/heading&gt;
+&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;“statement of findings and declaration of purpose&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1001"&gt;“&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 1001. &lt;/num&gt;
+&lt;chapeau class="inline"&gt;The Congress finds and declares that—&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s2996"&gt;42 USC 2996&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;&lt;/chapeau&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;“(1) &lt;/num&gt;
+&lt;content class="inline"&gt;there is a need to provide equal access to the system of justice in our Nation for individuals who seek redress of grievances;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;“(2) &lt;/num&gt;
+&lt;content class="inline"&gt;there is a need to provide high quality legal assistance to those who would be otherwise unable to afford adequate legal counsel and to continue the present vital legal services program;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;“(3) &lt;/num&gt;
+&lt;content class="inline"&gt;providing legal assistance to those who face an economic barrier to adequate legal counsel will serve best the ends of justice;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="4"&gt;“(4) &lt;/num&gt;
+&lt;content class="inline"&gt;for many of our citizens, the availability of legal services has reaffirmed faith in our government of laws;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="5"&gt;“(5) &lt;/num&gt;
+&lt;content class="inline"&gt;to preserve its strength, the legal services program must be kept free from the influence of or use by it of political pressures; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="6"&gt;“(6) &lt;/num&gt;
+&lt;content class="inline"&gt;attorneys providing legal assistance must have full freedom to protect the best interests of their clients in keeping with the Code of Professional Responsibility, the Canons of Ethics, and the high standards of the legal profession.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;“definitions&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1002"&gt;“&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 1002. &lt;/num&gt;
+&lt;chapeau class="inline"&gt;As used in this title, the term—&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s2996a"&gt;42 USC 2996a&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;&lt;/chapeau&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;“(1) &lt;/num&gt;
+&lt;content class="inline"&gt;‘Board’ means the Board of Directors of the Legal Services Corporation;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;“(2) &lt;/num&gt;
+&lt;content class="inline"&gt;‘Corporation’ means the Legal Services Corporation established under this title;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;“(3) &lt;/num&gt;
+&lt;content class="inline"&gt;‘eligible client’ means any person financially unable to afford legal assistance;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="4"&gt;“(4) &lt;/num&gt;
+&lt;content class="inline"&gt;‘Governor’ means the chief executive officer of a State;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="5"&gt;“(5) &lt;/num&gt;
+&lt;content class="inline"&gt;‘legal assistance’ means the provision of any legal services consistent with the purposes and provisions of this title;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>25401-26003</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>88 Stat. 446</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>88</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 2 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “District of Columbia Campaign&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;D.C. Code 1–1121 note.&lt;/p&gt;&lt;/sidenote&gt; Finance Reform and Conflict of Interest Act.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>29541-29547</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>88 Stat. 446</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>88</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 11 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “District of Columbia Campaign&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;D.C. Code 1–1121 note.&lt;/p&gt;&lt;/sidenote&gt; Finance Reform and Conflict of Interest Act.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>29541-29547</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>88 Stat. 446</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>88</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 6 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “District of Columbia Campaign&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;D.C. Code 1–1121 note.&lt;/p&gt;&lt;/sidenote&gt; Finance Reform and Conflict of Interest Act.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>29541-29547</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>88 Stat. 446</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>88</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 10 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “District of Columbia Campaign&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;D.C. Code 1–1121 note.&lt;/p&gt;&lt;/sidenote&gt; Finance Reform and Conflict of Interest Act.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>29541-29547</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>88 Stat. 446</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>88</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 8 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content class="inline"&gt;This Act may be cited as the “District of Columbia Campaign&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;D.C. Code 1–1121 note.&lt;/p&gt;&lt;/sidenote&gt; Finance Reform and Conflict of Interest Act.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>29541-29547</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>88 Stat. 823</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>88</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Multiple section tags — bare enacting &lt;section class="inline"&gt; at line 43826 (no num) collides with later "Sec. 1." GENERAL PROVISIONS at line 43872, because the null-SectionNumber fallback for the enacting section equals the numeric key for "Sec. 1."</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;enactingFormula&gt;&lt;i&gt;Be it enacted by the Senate and House of Representatives of the United States of America in Congress assembled,&lt;/i&gt;&lt;/enactingFormula&gt; &lt;section class="inline"&gt;&lt;chapeau class="inline"&gt;That the following &lt;sidenote&gt;&lt;p class="indent0 firstIndent1 fontsize8"&gt;District of Columbia Appropriation Act, 1975.&lt;/p&gt;&lt;/sidenote&gt; sums are appropriated, out of any money in the Treasury not otherwise appropriated, for the District of Columbia for the fiscal year ending June 30, 1975, and for other purposes, namely:&lt;/chapeau&gt;
+&lt;appropriations level="intermediate"&gt;&lt;heading&gt;Federal Payment to the District of Columbia&lt;/heading&gt;
+&lt;content&gt;For payment to the following funds of the District of Columbia for the fiscal year ending June 30, 1975: $221,200,000 to the general &lt;page identifier="/us/stat/88/823"&gt;88 &lt;inline class="smallCaps"&gt;Stat.&lt;/inline&gt; 823&lt;/page&gt; fund; $3,200,000 to the water fund; and $2,400,000 to the sanitary sewage works fund; as authorized by the District of Columbia Self-Government and Governmental Reorganization Act, Public Law 93–198; and the Act of May 18, 1954 (D.C. Code, 43–1541 and 1611).&lt;sidenote&gt;&lt;p class="indent0 firstIndent1 fontsize8"&gt;&lt;ref href="/us/dcc/1/121"&gt;D.C. Code 1–121&lt;/ref&gt; note.&lt;/p&gt;&lt;/sidenote&gt;&lt;/content&gt;
+</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>43826-43828</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>88 Stat. 1171</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>88</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 21 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;legislative findings and declaration of policy&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 2. &lt;/num&gt;
+&lt;content class="inline"&gt;
+&lt;p class="inline"&gt;Eggs constitute one of the basic, natural foods in the diet. &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t7/s2701"&gt;7 USC 2701&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; They are produced by many individual egg producers throughout the United States. Egg products, spent fowl, and products of spent fowl are derivatives of egg production. These products move in interstate and foreign commerce and those which do not move in such channels of commerce directly burden or affect interstate commerce of these products. The maintenance and expansion of existing markets and the development of new or improved markets and uses are vital to the welfare of egg producers and those concerned with marketing, using, and processing eggs as well as the general economy of the Nation. The production and marketing of these products by numerous individual egg producers have prevented the development and carrying out of adequate and coordinated programs of research and promotion necessary for the maintenance of markets and the development of new products of, and markets for, eggs, egg products, spent fowl, and products of spent fowl. Without an effective and coordinated method for assuring cooperative and collective action in providing for and financing such programs, individual egg producers are unable to provide, obtain, or carry out the research, consumer and producer information, and promotion necessary to maintain and improve markets for any or all of these products.&lt;/p&gt;
+&lt;p class="indent0 firstIndent1 fontsize10"&gt;It has long been recognized that it is in the public interest to provide an adequate, steady supply of fresh eggs readily available to the consumers of the Nation. Maintenance of markets and the development of new markets, both domestic and foreign, are essential to the egg industry if the consumers of eggs, egg products, spent fowl, or products of spent fowl are to be assured of an adequate, steady supply of such products.&lt;/p&gt;
+&lt;p class="indent0 firstIndent1 fontsize10"&gt;It is therefore declared to be the policy of the Congress and the purpose of this Act that it is essential and in the public interest, through the exercise of the powers provided herein, to authorize and enable the establishment of an orderly procedure for the development and the financing through an adequate assessment, an effective and continuous coordinated program of research, consumer and producer education, and promotion designed to strengthen the egg industry’s position in the marketplace, and maintain and expand domestic and foreign markets and uses for eggs, egg products, spent fowl, and products of spent fowl of the United States. Nothing in this Act shall be construed to mean, or provide for, control of production or otherwise limit the right of individual egg producers to produce commercial eggs.&lt;/p&gt;
+&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>57502-57512</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>88 Stat. 1233</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>88</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 2 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content&gt;This Act may be cited as the “Energy Reorganization Act of 1974”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s5801"&gt;42 USC 5801 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>59946-59953</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>88 Stat. 1233</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>88</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 10 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content&gt;This Act may be cited as the “Energy Reorganization Act of 1974”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s5801"&gt;42 USC 5801 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>59946-59953</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>88 Stat. 1233</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>88</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 9 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content&gt;This Act may be cited as the “Energy Reorganization Act of 1974”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s5801"&gt;42 USC 5801 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>59946-59953</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>88 Stat. 1233</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>88</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 12 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content&gt;This Act may be cited as the “Energy Reorganization Act of 1974”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s5801"&gt;42 USC 5801 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>59946-59953</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>88 Stat. 1263</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>88</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 4 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;limitations on contributions and expenditures&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;content&gt;Section 608 of title 18, United States Code, relating to limitations on contributions and expenditures, is amended by striking out subsections (b) and (c) and inserting in lieu thereof the following:
+&lt;quotedContent&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;“(b)&lt;/num&gt;
+&lt;paragraph class="inline"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content&gt;Except as otherwise provided by paragraphs (2) and (3), no person shall make contributions to any candidate with respect to any election for Federal office which, in the aggregate, exceed $1,000.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;“(2) &lt;/num&gt;
+&lt;content&gt;No political committee (other than a principal campaign committee) shall make contributions to any candidate with respect to any election for Federal office which, in the aggregate, exceed $5,000. Contributions by the national committee of a political party serving as the principal campaign committee of a candidate for the office of President of the United States shall not exceed the limitation imposed by the preceding sentence with respect to any other candidate for Federal office. For purposes of this paragraph, the term ‘political &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;“Political committee.”&lt;/p&gt;&lt;/sidenote&gt; committee’ means an organization registered as a political committee under section 303 of the Federal Election Campaign Act of 1971 for &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;i&gt;Post&lt;/i&gt;, p. 1276.&lt;/p&gt;&lt;/sidenote&gt; a period of not less than 6 months which has received contributions from more than 50 persons and, except for any State political party organization, has made contributions to 5 or more candidates for Federal office.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;“(3) &lt;/num&gt;
+&lt;content&gt;No individual shall make contributions aggregating more than $25,000 in any calendar year. For purposes of this paragraph, any contribution made in a year other than the calendar year in which the election is held with respect to which such contribution was made, is considered to be made during the calendar year in which such election is held.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="4"&gt;“(4) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;For purposes of this subsection—&lt;/chapeau&gt;
+&lt;subparagraph class="indent2 firstIndent1 fontsize10"&gt;
+&lt;num value="A"&gt;“(A) &lt;/num&gt;
+&lt;content&gt;contributions to a named candidate made to any political committee authorized by such candidate, in writing, to accept contributions on his behalf shall be considered to be contributions made to such candidate; and&lt;/content&gt;
+&lt;/subparagraph&gt;
+&lt;subparagraph class="indent2 firstIndent1 fontsize10"&gt;
+&lt;num value="B"&gt;“(B) &lt;/num&gt;
+&lt;content&gt;contributions made to or for the benefit of any candidate nominated by a political party for election to the office of Vice President of the United States shall be considered to be contributions made to or for the benefit of the candidate of such party for election to the office of President of the United States.&lt;/content&gt;
+&lt;/subparagraph&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="5"&gt;“(5) &lt;/num&gt;
+&lt;content&gt;The limitations imposed by paragraphs (1) and (2) of this subsection shall apply separately with respect to each election, except that all elections held in any calendar year for the office of President of the United States (except a general election for such office) shall be considered to be one election.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;page identifier="/us/stat/88/1264"&gt;88 &lt;inline class="smallCaps"&gt;Stat&lt;/inline&gt;. 1264&lt;/page&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="6"&gt;“(6) &lt;/num&gt;
+&lt;content&gt;For purpos
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>61501-61948</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>88 Stat. 1263</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>88</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 10 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;limitations on contributions and expenditures&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;content&gt;Section 608 of title 18, United States Code, relating to limitations on contributions and expenditures, is amended by striking out subsections (b) and (c) and inserting in lieu thereof the following:
+&lt;quotedContent&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;“(b)&lt;/num&gt;
+&lt;paragraph class="inline"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content&gt;Except as otherwise provided by paragraphs (2) and (3), no person shall make contributions to any candidate with respect to any election for Federal office which, in the aggregate, exceed $1,000.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;“(2) &lt;/num&gt;
+&lt;content&gt;No political committee (other than a principal campaign committee) shall make contributions to any candidate with respect to any election for Federal office which, in the aggregate, exceed $5,000. Contributions by the national committee of a political party serving as the principal campaign committee of a candidate for the office of President of the United States shall not exceed the limitation imposed by the preceding sentence with respect to any other candidate for Federal office. For purposes of this paragraph, the term ‘political &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;“Political committee.”&lt;/p&gt;&lt;/sidenote&gt; committee’ means an organization registered as a political committee under section 303 of the Federal Election Campaign Act of 1971 for &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;i&gt;Post&lt;/i&gt;, p. 1276.&lt;/p&gt;&lt;/sidenote&gt; a period of not less than 6 months which has received contributions from more than 50 persons and, except for any State political party organization, has made contributions to 5 or more candidates for Federal office.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;“(3) &lt;/num&gt;
+&lt;content&gt;No individual shall make contributions aggregating more than $25,000 in any calendar year. For purposes of this paragraph, any contribution made in a year other than the calendar year in which the election is held with respect to which such contribution was made, is considered to be made during the calendar year in which such election is held.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="4"&gt;“(4) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;For purposes of this subsection—&lt;/chapeau&gt;
+&lt;subparagraph class="indent2 firstIndent1 fontsize10"&gt;
+&lt;num value="A"&gt;“(A) &lt;/num&gt;
+&lt;content&gt;contributions to a named candidate made to any political committee authorized by such candidate, in writing, to accept contributions on his behalf shall be considered to be contributions made to such candidate; and&lt;/content&gt;
+&lt;/subparagraph&gt;
+&lt;subparagraph class="indent2 firstIndent1 fontsize10"&gt;
+&lt;num value="B"&gt;“(B) &lt;/num&gt;
+&lt;content&gt;contributions made to or for the benefit of any candidate nominated by a political party for election to the office of Vice President of the United States shall be considered to be contributions made to or for the benefit of the candidate of such party for election to the office of President of the United States.&lt;/content&gt;
+&lt;/subparagraph&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="5"&gt;“(5) &lt;/num&gt;
+&lt;content&gt;The limitations imposed by paragraphs (1) and (2) of this subsection shall apply separately with respect to each election, except that all elections held in any calendar year for the office of President of the United States (except a general election for such office) shall be considered to be one election.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;page identifier="/us/stat/88/1264"&gt;88 &lt;inline class="smallCaps"&gt;Stat&lt;/inline&gt;. 1264&lt;/page&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="6"&gt;“(6) &lt;/num&gt;
+&lt;content&gt;For purpos
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>61501-61948</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>88 Stat. 1263</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>88</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 2 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;limitations on contributions and expenditures&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;content&gt;Section 608 of title 18, United States Code, relating to limitations on contributions and expenditures, is amended by striking out subsections (b) and (c) and inserting in lieu thereof the following:
+&lt;quotedContent&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;“(b)&lt;/num&gt;
+&lt;paragraph class="inline"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content&gt;Except as otherwise provided by paragraphs (2) and (3), no person shall make contributions to any candidate with respect to any election for Federal office which, in the aggregate, exceed $1,000.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;“(2) &lt;/num&gt;
+&lt;content&gt;No political committee (other than a principal campaign committee) shall make contributions to any candidate with respect to any election for Federal office which, in the aggregate, exceed $5,000. Contributions by the national committee of a political party serving as the principal campaign committee of a candidate for the office of President of the United States shall not exceed the limitation imposed by the preceding sentence with respect to any other candidate for Federal office. For purposes of this paragraph, the term ‘political &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;“Political committee.”&lt;/p&gt;&lt;/sidenote&gt; committee’ means an organization registered as a political committee under section 303 of the Federal Election Campaign Act of 1971 for &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;i&gt;Post&lt;/i&gt;, p. 1276.&lt;/p&gt;&lt;/sidenote&gt; a period of not less than 6 months which has received contributions from more than 50 persons and, except for any State political party organization, has made contributions to 5 or more candidates for Federal office.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;“(3) &lt;/num&gt;
+&lt;content&gt;No individual shall make contributions aggregating more than $25,000 in any calendar year. For purposes of this paragraph, any contribution made in a year other than the calendar year in which the election is held with respect to which such contribution was made, is considered to be made during the calendar year in which such election is held.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="4"&gt;“(4) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;For purposes of this subsection—&lt;/chapeau&gt;
+&lt;subparagraph class="indent2 firstIndent1 fontsize10"&gt;
+&lt;num value="A"&gt;“(A) &lt;/num&gt;
+&lt;content&gt;contributions to a named candidate made to any political committee authorized by such candidate, in writing, to accept contributions on his behalf shall be considered to be contributions made to such candidate; and&lt;/content&gt;
+&lt;/subparagraph&gt;
+&lt;subparagraph class="indent2 firstIndent1 fontsize10"&gt;
+&lt;num value="B"&gt;“(B) &lt;/num&gt;
+&lt;content&gt;contributions made to or for the benefit of any candidate nominated by a political party for election to the office of Vice President of the United States shall be considered to be contributions made to or for the benefit of the candidate of such party for election to the office of President of the United States.&lt;/content&gt;
+&lt;/subparagraph&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="5"&gt;“(5) &lt;/num&gt;
+&lt;content&gt;The limitations imposed by paragraphs (1) and (2) of this subsection shall apply separately with respect to each election, except that all elections held in any calendar year for the office of President of the United States (except a general election for such office) shall be considered to be one election.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;page identifier="/us/stat/88/1264"&gt;88 &lt;inline class="smallCaps"&gt;Stat&lt;/inline&gt;. 1264&lt;/page&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;num value="6"&gt;“(6) &lt;/num&gt;
+&lt;content&gt;For purpos
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>61501-61948</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>88 Stat. 1364</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>88</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>93 Session 1</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 5 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content&gt;This&lt;sidenote&gt;&lt;p class="indent0 firstIndent0 fontsize8"&gt;&lt;ref href="/us/usc/t12/s1723e"&gt;12 USC 1723e note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; Act may be cited as the “&lt;shortTitle role="act"&gt;Emergency Home Purchase Assistance Act of 1974&lt;/shortTitle&gt;”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>75439-75445</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>88 Stat. 1376</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>88</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>93 Session 1</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 13 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content&gt;This&lt;sidenote&gt;&lt;p class="indent0 firstIndent0 fontsize8"&gt;&lt;ref href="/us/usc/t16/s838"&gt;16 USC 838 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; Act may be cited as the “&lt;shortTitle role="act"&gt;Federal Columbia River Transmission System Act&lt;/shortTitle&gt;”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>76158-76164</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>88 Stat. 1422</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>88</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>93 Session 1</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 3 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content&gt;This Act may be cited as the “&lt;shortTitle role="act"&gt;District of Columbia Public&lt;sidenote&gt;&lt;p class="indent0 firstIndent0 fontsize8"&gt;&lt;ref href="/us/dcc/31/1701"&gt;D.C. Code 31–1701 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; Postsecondary Education Reorganization Act&lt;/shortTitle&gt;”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>78736-78742</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>88 Stat. 1422</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>88</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>93 Session 1</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 9 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content&gt;This Act may be cited as the “&lt;shortTitle role="act"&gt;District of Columbia Public&lt;sidenote&gt;&lt;p class="indent0 firstIndent0 fontsize8"&gt;&lt;ref href="/us/dcc/31/1701"&gt;D.C. Code 31–1701 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; Postsecondary Education Reorganization Act&lt;/shortTitle&gt;”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>78736-78742</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>88 Stat. 1422</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>88</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>93 Session 1</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 7 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content&gt;This Act may be cited as the “&lt;shortTitle role="act"&gt;District of Columbia Public&lt;sidenote&gt;&lt;p class="indent0 firstIndent0 fontsize8"&gt;&lt;ref href="/us/dcc/31/1701"&gt;D.C. Code 31–1701 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; Postsecondary Education Reorganization Act&lt;/shortTitle&gt;”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>78736-78742</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>88 Stat. 1431</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>88</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>93 Session 1</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 17 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;heading class="smallCaps centered"&gt;declaration of findings and policy&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 2. &lt;/num&gt;
+&lt;subsection class="inline"&gt;&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;chapeau&gt;The Congress hereby finds that&lt;sidenote&gt;&lt;p class="indent0 firstIndent0 fontsize8"&gt;&lt;ref href="/us/usc/t42/s5551"&gt;42 USC 5551&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;—&lt;/chapeau&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content&gt;the needs of a viable society depend on an ample supply of energy;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content&gt;the current imbalance between domestic supply and demand for fuels and energy is likely to persist for some time;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="3"&gt;(3) &lt;/num&gt;
+&lt;content&gt;dependence on nonrenewable energy resources cannot be continued indefinitely, particularly at current rates of consumption;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="4"&gt;(4) &lt;/num&gt;
+&lt;content&gt;it is in the Nation’s interest to expedite the long-term development of renewable and nonpolluting energy resources, such as solar energy;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="5"&gt;(5) &lt;/num&gt;
+&lt;content&gt;the various solar energy technologies are today at widely differing stages of development, with some already near the stage of commercial application and others still requiring basic research;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="6"&gt;(6) &lt;/num&gt;
+&lt;content&gt;the early development and export of viable equipment utilizing solar energy, consistent with the established preeminence of the United States in the field of high technology products, can make a valuable contribution to our balance of trade;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="7"&gt;(7) &lt;/num&gt;
+&lt;content&gt;the mass production and use of equipment utilizing solar energy will help to eliminate the dependence of the United States upon foreign energy sources and promote the national defense;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="8"&gt;(8) &lt;/num&gt;
+&lt;content&gt;to date, the national effort in research, development, and demonstration activities relating to the utilization of solar energy has been extremely limited; therefore&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="9"&gt;(9) &lt;/num&gt;
+&lt;content&gt;the urgency of the Nation’s critical energy shortages and the need to make clean and renewable energy alternatives commercially viable require that the Nation undertake an intensive research, development, and demonstration program with an estimated Federal investment which may reach or exceed $1,000,000,000.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;/subsection&gt;
+&lt;subsection class="indent0 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;chapeau&gt;The Congress declares that it is the policy of the Federal Government to—&lt;/chapeau&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content&gt;pursue a vigorous and viable program of research and resource assessment of solar energy as a major source of energy for our national needs; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content&gt;provide for the development and demonstration of practicable means to employ solar energy on a commercial scale.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;/subsection&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>79204-79260</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>88 Stat. 1439</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>88</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>93 Session 1</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 15 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;heading class="smallCaps centered"&gt;authorizations of appropriations&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 2. &lt;/num&gt;
+&lt;subsection class="inline"&gt;&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;chapeau&gt;There are authorized to be appropriated for the Department&lt;sidenote&gt;&lt;p class="indent0 firstIndent0 fontsize8"&gt;&lt;ref href="/us/usc/t22/s901a note"&gt;22 USC 901a note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; of State for fiscal year 1975, to carry out the authorities, functions, duties, and responsibilities in the conduct of the foreign affairs of the United States, including trade negotiations, and other purposes authorized by law, the following amounts:&lt;/chapeau&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content&gt;for the “Administration of Foreign Affairs”, $370,045,000;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content&gt;for “International Organizations and Conferences”, $229,604,000;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="3"&gt;(3) &lt;/num&gt;
+&lt;content&gt;for “International Commissions”, $17,832,000;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="4"&gt;(4) &lt;/num&gt;
+&lt;content&gt;for “Educational Exchange”, $75,000,000; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="5"&gt;(5) &lt;/num&gt;
+&lt;content&gt;for “Migration and Refugee Assistance”, $9,420,000.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;/subsection&gt;
+&lt;subsection class="indent0 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;chapeau&gt;There are authorized to be appropriated for the United States Information Agency for fiscal year 1975, to carry out international informational activities and programs under the United States Information and Educational Exchange Act of 1948, the Mutual&lt;sidenote&gt;&lt;p class="indent0 firstIndent0 fontsize8"&gt;&lt;ref href="/us/usc/t22/s1431 note"&gt;22 USC 1431 note&lt;/ref&gt;.&lt;/p&gt;&lt;p class="indent0 firstIndent0 fontsize8"&gt;&lt;ref href="/us/usc/t22/s2451 note"&gt;22 USC 2451 note&lt;/ref&gt;.&lt;/p&gt;&lt;p class="indent0 firstIndent0 fontsize8"&gt;&lt;ref href="/us/usc/t22/s1461 note"&gt;22 USC 1461 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; Education and Cultural Exchange Act of 1941, and Reorganization Plan Numbered 8 of 1953, and other purposes authorized by law, the following amounts:&lt;/chapeau&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content&gt;for “Salaries and Expenses” and “Salaries and Expenses (special foreign currency program)”, $228,368,000, except that so much of such amount as may be appropriated for “Salaries and Expenses (special foreign currency program)” may be appropriated without fiscal year limitation;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content&gt;for “Special International Exhibitions”, $6,770,000; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 fontsize10"&gt;
+&lt;num value="3"&gt;(3) &lt;/num&gt;
+&lt;content&gt;for “Acquisition and Construction of Radio Facilities”, $4,400,000.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;/subsection&gt;
+&lt;subsection class="indent0 fontsize10"&gt;
+&lt;num value="c"&gt;(c) &lt;/num&gt;
+&lt;content&gt;In addition to amounts otherwise authorized, there are authorized to be appropriated to the Secretary of State for the fiscal year 1975 not to exceed $40,000,000 to carry out the provisions of section 101(b) of the Foreign Relations Authorization Act of 1972, relating&lt;sidenote&gt;&lt;p class="indent0 firstIndent0 fontsize8"&gt;&lt;ref href="/us/stat/86/489"&gt;86 Stat. 489&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; to Soviet refugee assistance.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="indent0 fontsize10"&gt;
+&lt;num value="d"&gt;(d) &lt;/num&gt;
+&lt;content&gt;In addition to amounts authorized in subsections (a) and (b) of this section, there are authorized to be appropriated for fiscal year 1975 for the Department of State and for the United States Information Agency such additional amounts as may be necessary for increases in salary, pay, retirement, and other employee benefits authorized by law which arise subsequent to the date of
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>79853-79909</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>88 Stat. 1784</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>88</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 4 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;purpose&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content&gt;For the purpose of preserving and protecting for public&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t16/s460ff"&gt;16 USC 460ff&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; use and enjoyment, the historic, scenic, natural, and recreational values of the Cuyahoga River and the adjacent lands of the Cuyahoga Valley and for the purpose of providing for the maintenance of needed recreational open space necessary to the urban environment, the Cuyahoga Valley National Recreation Area, hereafter referred to as the “recreation area”, shall be established within six months after the date of enactment of this Act. In the management of the recreation area, the Secretary of the Interior (hereafter referred to as the “Secretary”) shall utilize the recreation area resources in a manner which will preserve its scenic, natural, and historic setting while providing for the recreational and educational needs of the visiting public.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>94853-94859</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>88 Stat. 1789</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>88</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 9 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;declaration of purpose&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;content&gt;The Congress hereby finds that Federal information &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t44/s3501"&gt;44 USC 3501 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; reporting requirements have placed an unprecedented paperwork burden upon private citizens, recipients of Federal assistance, businesses, governmental contractors, and State and local governments.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;content&gt;The Congress hereby affirms that it is the policy of the Federal Government to minimize the information reporting burden, consistent with its needs for information to set policy and operate its lawful programs.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="c"&gt;(c) &lt;/num&gt;
+&lt;content&gt;The Congress hereby determines that a renewed effort is required to assure that this policy is fully implemented and that it is necessary to reexamine the policies and procedures of the Federal Government which have an impact on the paperwork burden for the purpose of ascertaining what changes are necessary and desirable in its information policies and practices.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>95068-95085</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>88 Stat. 1795</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>88</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 56 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;food and nutrition&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 2. &lt;/num&gt;
+&lt;chapeau class="inline"&gt;Section 103 of the Foreign Assistance Act of 1961 is &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t22/s2151a"&gt;22 USC 2151a&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; amended—&lt;/chapeau&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;content&gt;by inserting the subsection designation “&lt;quotedText&gt;(a)&lt;/quotedText&gt;” immediately before “&lt;quotedText&gt;In&lt;/quotedText&gt;” ;&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content&gt;by striking out “&lt;quotedText&gt;$291,000,000 for each of the fiscal years 1974 and 1975&lt;/quotedText&gt;” and inserting in lieu thereof “&lt;quotedText&gt;$291,000,000 for the fiscal year 1974, and $500,000,000 for the fiscal year 1975&lt;/quotedText&gt;”; and&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;(3) &lt;/num&gt;
+&lt;content&gt;by adding at the end thereof the following:&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent0 firstIndent1 fontsize10"&gt;
+&lt;quotedContent&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;“(b) &lt;/num&gt;
+&lt;content&gt;The Congress finds that, due to rising world food, fertilizer, and petroleum costs, human suffering and deprivation are growing in the poorest and most slowly developing countries. The greatest potential for significantly expanding world food production at relatively low cost lies in increasing the productivity of small farmers who constitute a majority of the nearly one billion people living in those countries. Increasing the emphasis on rural development and expanded food production in the poorest nations of the developing world is a matter of social justice as well as an important factor in slowing the rate of inflation in the industrialized countries. In the allocation of funds under this section, special attention should be given to increasing agricultural production in the countries with per capita incomes under $300 a year and which are the most severely affected by sharp increases in worldwide commodity prices.”&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;/quotedContent&gt;
+&lt;/paragraph&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>95473-95499</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>88 Stat. 1845</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>88</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 7 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;emergency job programs authorized&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content&gt;The Comprehensive Employment and Training Act of 1973 is amended by redesignating title VI, and all references thereto, &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t29/s981–992/801"&gt;29 USC 981–992, 801 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; as title VII, by redesignating sections 601 through 615, and all references thereto, as sections 701 through 715, respectively, and by inserting after title V the following new title:
+&lt;quotedContent&gt;
+&lt;title&gt;
+&lt;num value="VI"&gt;“TITLE VI—&lt;/num&gt;
+&lt;heading class="inline"&gt;EMERGENCY JOB PROGRAMS&lt;/heading&gt;
+&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;“authorization of appropriations&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="601"&gt;“&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 601. &lt;/num&gt;
+&lt;content&gt;There are authorized to be appropriated $2,500,000,000 &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t29/s961"&gt;29 USC 961&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; for fiscal year 1975 for carrying out the provisions of this title. Any amounts so appropriated for such fiscal year which are not obligated prior to the end of such fiscal year shall remain available for obligation until December 31, 1975.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;“financial assistance&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="602"&gt;“&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 602. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;content&gt;The Secretary shall enter into arrangements with &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t29/s962"&gt;29 USC 962&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;eligible applicants in accordance with the provisions of this title in order to make financial assistance available for the purpose of providing transitional employment, for unemployed and underemployed persons in jobs providing needed public services, and training and manpower services related to such employment which are otherwise unavailable, and enabling such persons to move into employment not supported under this Act.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;“(b) &lt;/num&gt;
+&lt;content&gt;Not less than 90 per centum of the funds appropriated pursuant to this title which are used by an eligible applicant for public service employment programs shall be expended only for wages and employment benefits to persons employed in public service jobs pursuant to this title.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="c"&gt;“(c) &lt;/num&gt;
+&lt;content&gt;The provisions of section 204(d) and sections 205 through 211 &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t29/s844–851"&gt;29 USC 844–851&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; shall apply to financial assistance under this title.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="d"&gt;“(d) &lt;/num&gt;
+&lt;content&gt;In filling public service jobs with financial assistance under this title, eligible applicants shall give preferred consideration, to the maximum extent feasible and consistent with other provisions of this Act, to unemployed persons who have exhausted unemployment insurance benefits, to unemployed persons who are not eligible for unemployment insurance benefits (except for persons lacking work experience), and to unemployed persons who have been unemployed for fifteen or more weeks.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="e"&gt;“(e) &lt;/num&gt;
+&lt;content&gt;For purposes of this section, the term ‘eligible applicants’&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;“Eligible applicants.”&lt;/p&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t29/s811"&gt;29 USC 811&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; means prime sponsors qualified under title I and Indian tribes on Federal or State reservations.&lt;/content&gt;
+&lt;/subsection&gt;
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>97898-98025</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>88 Stat. 1845</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>88</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 10 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;emergency job programs authorized&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content&gt;The Comprehensive Employment and Training Act of 1973 is amended by redesignating title VI, and all references thereto, &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t29/s981–992/801"&gt;29 USC 981–992, 801 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; as title VII, by redesignating sections 601 through 615, and all references thereto, as sections 701 through 715, respectively, and by inserting after title V the following new title:
+&lt;quotedContent&gt;
+&lt;title&gt;
+&lt;num value="VI"&gt;“TITLE VI—&lt;/num&gt;
+&lt;heading class="inline"&gt;EMERGENCY JOB PROGRAMS&lt;/heading&gt;
+&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;“authorization of appropriations&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="601"&gt;“&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 601. &lt;/num&gt;
+&lt;content&gt;There are authorized to be appropriated $2,500,000,000 &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t29/s961"&gt;29 USC 961&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; for fiscal year 1975 for carrying out the provisions of this title. Any amounts so appropriated for such fiscal year which are not obligated prior to the end of such fiscal year shall remain available for obligation until December 31, 1975.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;“financial assistance&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="602"&gt;“&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 602. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;content&gt;The Secretary shall enter into arrangements with &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t29/s962"&gt;29 USC 962&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;eligible applicants in accordance with the provisions of this title in order to make financial assistance available for the purpose of providing transitional employment, for unemployed and underemployed persons in jobs providing needed public services, and training and manpower services related to such employment which are otherwise unavailable, and enabling such persons to move into employment not supported under this Act.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;“(b) &lt;/num&gt;
+&lt;content&gt;Not less than 90 per centum of the funds appropriated pursuant to this title which are used by an eligible applicant for public service employment programs shall be expended only for wages and employment benefits to persons employed in public service jobs pursuant to this title.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="c"&gt;“(c) &lt;/num&gt;
+&lt;content&gt;The provisions of section 204(d) and sections 205 through 211 &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t29/s844–851"&gt;29 USC 844–851&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; shall apply to financial assistance under this title.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="d"&gt;“(d) &lt;/num&gt;
+&lt;content&gt;In filling public service jobs with financial assistance under this title, eligible applicants shall give preferred consideration, to the maximum extent feasible and consistent with other provisions of this Act, to unemployed persons who have exhausted unemployment insurance benefits, to unemployed persons who are not eligible for unemployment insurance benefits (except for persons lacking work experience), and to unemployed persons who have been unemployed for fifteen or more weeks.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="e"&gt;“(e) &lt;/num&gt;
+&lt;content&gt;For purposes of this section, the term ‘eligible applicants’&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;“Eligible applicants.”&lt;/p&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t29/s811"&gt;29 USC 811&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; means prime sponsors qualified under title I and Indian tribes on Federal or State reservations.&lt;/content&gt;
+&lt;/subsection&gt;
+…&lt;TRUNCATED&gt;</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>97898-98025</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>88 Stat. 1869</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>88</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 8 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="101"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 101. &lt;/num&gt;
+&lt;content&gt;This Act may be cited as the “Emergency Unemployment Compensation Act of 1974”. &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t26/s3304"&gt;26 USC 3304 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>99423-99429</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>88 Stat. 1873</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>88</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 8 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;establishment and purpose of commission&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="201"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 201. &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;content&gt;There is hereby created in the Library of Congress &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t17/s201"&gt;17 USC 201 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; a National Commission on New Technological Uses of Copyrighted Works (hereafter called the Commission).&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;The purpose of the Commission is to study and compile data on:&lt;/chapeau&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;(1) &lt;/num&gt;
+&lt;chapeau class="inline"&gt;the reproduction and use of copyrighted works of authorship—&lt;/chapeau&gt;
+&lt;subparagraph class="indent2 firstIndent1 fontsize10"&gt;
+&lt;num value="A"&gt;(A) &lt;/num&gt;
+&lt;content&gt;in conjunction with automatic systems capable of storing, processing, retrieving, and transferring information, and&lt;/content&gt;
+&lt;/subparagraph&gt;
+&lt;subparagraph class="indent2 firstIndent1 fontsize10"&gt;
+&lt;num value="B"&gt;(B) &lt;/num&gt;
+&lt;content&gt;by various forms of machine reproduction, not including reproduction by or at the request of instructors for use in face-to-face teaching activities; and&lt;/content&gt;
+&lt;/subparagraph&gt;
+&lt;/paragraph&gt;
+&lt;paragraph class="indent1 firstIndent1 fontsize10"&gt;
+&lt;num value="2"&gt;(2) &lt;/num&gt;
+&lt;content&gt;the creation of new works by the application or intervention of such automatic systems or machine reproduction.&lt;/content&gt;
+&lt;/paragraph&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="c"&gt;(c) &lt;/num&gt;
+&lt;content&gt;The Commission shall make recommendations as to such changes&lt;page identifier="/us/stat/88/1874"&gt;88 &lt;inline class="smallCaps"&gt;Stat&lt;/inline&gt;. 1874&lt;/page&gt; in copyright law or procedures that may be necessary to assure for such purposes access to copyrighted works, and to provide recognition of the rights of copyright owners.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>99770-99803</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>88 Stat. 1878</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>88</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 16 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;short title&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;content&gt;This Act may be cited as the “Federal Nonnuclear Energy Research and Development Act of 1974”.&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t42/s5901"&gt;42 USC 5901 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt;&lt;/content&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>100128-100134</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>88 Stat. 1910</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>88</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 7 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section&gt;
+&lt;heading class="smallCaps centered"&gt;powers or the commission&lt;/heading&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="3"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 3 &lt;/num&gt;
+&lt;subsection class="inline"&gt;
+&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;content&gt;The Commission or, on authorization of the Commission, &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t25/s174"&gt;25 USC 174 note&lt;/ref&gt;.&lt;/p&gt;&lt;/sidenote&gt; any committee of two or more members is authorized, for the purposes of carrying out the provisions of this resolution, to sit and act at such places and times during the sessions, recesses, and adjourned periods of Congress, to require by subpena or otherwise the attendance of such witnesses and the production of such books, papers, and documents, to administer such oaths and affirmations, to take such testimony, to procure such printing and binding, and to make such expenditures, as it deems advisable. The Commission may make such rules respecting its organization and procedures as it deems necessary, except that no recommendation shall be reported from the Commission unless a majority of the Commission assent. Upon the authorization of the Commission subpenas may be issued over the signature of the Chairman of the Commission or of any member designated by him or the Commission, and may be served by such person or persons as may be designated by such Chairman or member. The Chairman of the Commission or any member thereof may administer oaths or affirmations to witnesses.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="b"&gt;(b) &lt;/num&gt;
+&lt;content&gt;The provisions of sections 192 through 194, inclusive, of title 2, United States Code, shall apply in the case of any failure of any witness to comply with any subpena when summoned under this section.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="c"&gt;(c) &lt;/num&gt;
+&lt;content&gt;The Commission is authorized to secure from any department, agency, or instrumentality of the executive branch of the Government any information it deems necessary to carry out its functions under this resolution and each such department, agency, or instrumentality is authorized and directed to furnish such information to the Commission and to conduct such studies and surveys as may be requested by the Chairman or the Vice Chairman when acting as Chairman.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;subsection class="firstIndent1 fontsize10"&gt;
+&lt;num value="d"&gt;(d) &lt;/num&gt;
+&lt;content&gt;If the Commission requires of any witness or of any Government &lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;Confidential materials.&lt;/p&gt;&lt;/sidenote&gt; agency the production of any materials which have theretofore been submitted to a Government agency on a confidential basis, and the confidentiality of those materials is protected by statute, the material so produced shall be held in confidence by the Commission.&lt;/content&gt;
+&lt;/subsection&gt;
+&lt;/section&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>102164-102185</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>88 Stat. 1975</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>88</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>93 Session 2</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Multiple section tags without num components — 2 sibling sections in this pLaw collapse to the same UniqueKey because the section elements have no num attribute directly under them</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Section tags should carry the "num" attribute directly (e.g. &lt;num value="1"&gt;Section 1.&lt;/num&gt;), or remove the redundant outer section wrapper so the numbered inner section becomes the top-level section.</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;section class="inline"&gt;
+&lt;content class="inline fontsize10"&gt;That chapter 31&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;Department of Justice.&lt;/p&gt;&lt;p class="firstIndent1 fontsize8"&gt;Working capital fund, establishment.&lt;/p&gt;&lt;/sidenote&gt; of title 28, United States Code, is amended by inserting the following new section at the end thereof:
+&lt;quotedContent&gt;
+&lt;section class="fontsize10"&gt;
+&lt;num value="527"&gt;“§ 527. &lt;/num&gt;
+&lt;heading&gt;Establishment of working capital fund&lt;/heading&gt;&lt;sidenote&gt;&lt;p class="firstIndent1 fontsize8"&gt;&lt;ref href="/us/usc/t28/s527"&gt;28 USC 527.&lt;/ref&gt;&lt;/p&gt;&lt;/sidenote&gt;
+&lt;content&gt;“There is hereby authorized to be established a working capital fund for the Department of Justice, which shall be available, without fiscal year limitation, for expenses and equipment necessary for maintenance and operations of such administrative services as the Attorney Genera], with the approval of the Office of Management and Budget, determines may be performed more advantageously as central services. The capital of the fund shall consist of the amount of the fair and reasonable value of such inventories, equipment, and other assets and inventories on order pertaining to the services to be carried on by the fund as the Attorney General may transfer to the fund less related liabilities and unpaid obligations together with any appropriations made for the purpose of providing capital. The fund shall be reimbursed or credited with advance payments from applicable appropriations and funds of the Department of Justice, other Federal agencies, and other sources authorized by law for supplies, materials, and services at rates which will recover the expenses of operations including accrual of annual leave and depreciation of plant and equipment of the fund. The fund shall also be credited with other receipts from sale or exchange of property or in payment for loss or damage to property held by the fund. There shall be transferred into the Treasury as miscellaneous receipts, as of the close of each fiscal year, any net income after making provisions for prior year losses, if any.&lt;/content&gt;
+&lt;/section&gt;
+&lt;/quotedContent&gt;
+&lt;/content&gt;
+&lt;/section&gt;
+</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>106416-106426</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>84 Stat. 2080-1</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>89</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>91 Session 1</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Public Law 91-696 (84 Stat. 2080-1) appears at the start of the vol 89 XML file but belongs in vol 84</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Move this pLaw out of STATUTE-89.xml and into STATUTE-84.xml. The law was approved Dec. 25, 1970 and its own Statutes citation reads 84 Stat. 2080-1, confirming vol 84 is the correct volume.</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>&lt;docNumber&gt;696&lt;/docNumber&gt;
+&lt;citableAs&gt;Public Law 91–696&lt;/citableAs&gt;
+&lt;citableAs&gt;84 Stat. 2080–1&lt;/citableAs&gt;
+&lt;approvedDate&gt;1970-12-25&lt;/approvedDate&gt;
+&lt;congress&gt;91&lt;/congress&gt;
+&lt;session&gt;1&lt;/session&gt;</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>&lt;statutesAtLarge&gt;
+ &lt;main&gt;
+  &lt;collection&gt;
+   &lt;component&gt;
+    &lt;publicLaws&gt;
+     &lt;component&gt;
+      &lt;pLaw&gt;</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>754-1038</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>89 Stat. 2-1</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>89</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>93 Session 1</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Reviewed: gap - no correction needed</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Legitimate volume-boundary quirk - PL 93-650 (a late-passed 93rd Congress joint resolution approved Jan. 4, 1974) is correctly printed in vol 89 with pagination 89 Stat. 2-1. The prefilter flagged a sequence gap (from 91-696 to 93-650) only because the preceding pLaw in this XML file is a misfiled 91-696. No misnumbering here.</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>&lt;docNumber&gt;650&lt;/docNumber&gt;
+&lt;citableAs&gt;Public Law 93–650&lt;/citableAs&gt;
+&lt;citableAs&gt;89 Stat. 2–1&lt;/citableAs&gt;
+&lt;approvedDate&gt;1974-01-04&lt;/approvedDate&gt;
+&lt;congress&gt;93&lt;/congress&gt;
+&lt;session&gt;1&lt;/session&gt;</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>&lt;statutesAtLarge&gt;
+ &lt;main&gt;
+  &lt;collection&gt;
+   &lt;component&gt;
+    &lt;publicLaws&gt;
+     &lt;component&gt;
+      &lt;pLaw&gt;</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>1044-1122</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>89 Stat. 3</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>89</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>94 Session 1</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Reviewed: gap - no correction needed</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Legitimate Congress-boundary - PL 94-1 is the first law of the new 94th Congress. The prefilter flagged the gap from 93-651 to 94-1 only because numbering resets across Congresses. No misnumbering here.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>&lt;docNumber&gt;1&lt;/docNumber&gt;
+&lt;citableAs&gt;Public Law 94–1&lt;/citableAs&gt;
+&lt;citableAs&gt;89 Stat. 3&lt;/citableAs&gt;
+&lt;approvedDate&gt;1975-01-24&lt;/approvedDate&gt;
+&lt;congress&gt;94&lt;/congress&gt;
+&lt;session&gt;1&lt;/session&gt;</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>&lt;statutesAtLarge&gt;
+ &lt;main&gt;
+  &lt;collection&gt;
+   &lt;component&gt;
+    &lt;publicLaws&gt;
+     &lt;component&gt;
+      &lt;pLaw&gt;</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>2075-2120</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>89 Stat. 26</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>89</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>94 Session 1</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Two sibling section elements within the same Act both numbered Sec. 601</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>The second section under TITLE VI (heading "Treatment for purposes of the investment credit of certain property used in international or territorial waters") should be Sec. 602, not Sec. 601 - a Sec. 601 already exists immediately above it (heading "Limitations on foreign tax credit for taxes paid in connection with foreign oil and gas income"). The "num" element on the second section should read Sec. 602.</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;num value="601"&gt;SEC. 601. &lt;/num&gt;
+&lt;heading&gt;LIMITATIONS ON FOREIGN TAX CREDIT FOR TAXES PAID IN CONNECTION WITH FOREIGN OIL AND GAS INCOME.&lt;/heading&gt;
+...
+&lt;/section&gt;
+&lt;section&gt;
+&lt;num value="601"&gt;SEC. 601. &lt;/num&gt;
+&lt;heading&gt;TREATMENT FOR PURPOSES OF THE INVESTMENT CREDIT OF CERTAIN PROPERTY USED IN INTERNATIONAL OR TERRITORIAL WATERS.&lt;/heading&gt;
+...
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;title&gt;
+   &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>5308-6128</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>89 Stat. 68</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>89</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>94 Session 1</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Unnumbered short-title section sibling collapses to same key as Sec. 1</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>The opening short-title clause ("That this Act may be cited as the 'National Insurance Development Act of 1975'") is wrapped in its own "section" sibling with no "num" child, then a separate "section" with num value="1" immediately follows containing the substantive findings. These two should be merged into a single Sec. 1 in the XML, or the short-title clause should be hoisted out of "section" altogether (e.g. into a "shortTitle" wrapper directly under main), so that Sec. 1's UniqueKey does not collide with the unnumbered preamble.</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>&lt;section class="inline"&gt;
+&lt;content class="inline"&gt;That this Act may be cited as the “&lt;shortTitle role="act"&gt;National Insurance Development Act of 1975&lt;/shortTitle&gt;”.&lt;/content&gt;
+&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="1"&gt;&lt;inline class="smallCaps"&gt;Section&lt;/inline&gt; 1. &lt;/num&gt;
+&lt;subsection class="inline"&gt;&lt;num value="a"&gt;(a) &lt;/num&gt;
+&lt;content&gt;The Congress finds that ...&lt;/content&gt;
+&lt;/subsection&gt;
+...
+&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>6288-6300</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>89 Stat. 611</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>89</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>94 Session 1</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Two sibling appropriations elements share identical heading "disaster loan fund"</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>TITLE V contains two sibling appropriations elements both with heading "Disaster loan fund" under the Small Business Administration - one establishing the fund's borrowing authority, the second adding $100,000,000 of additional capital. These are legitimate sibling appropriations (regular plus supplemental) but their identical heading makes the heading-derived Division UniqueKey collapse. This is the same pattern covered by an existing approved extractor-code correction (active correction #5 from vol 78).</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>&lt;appropriations level="small"&gt;
+&lt;heading&gt;disaster loan fund&lt;/heading&gt;
+&lt;content&gt;The Small Business Administration is hereby authorized to make such expenditures, within the limits of funds and borrowing authority available to the following funds ...&lt;/content&gt;
+&lt;/appropriations&gt;
+&lt;appropriations level="small"&gt;
+&lt;heading&gt;disaster loan fund&lt;/heading&gt;
+&lt;content&gt;For additional capital for the “Disaster loan fund”, authorized by the Small Business Act, as amended, $100,000,000, to remain available without fiscal year limitation, for the non-physical disaster loan program.&lt;/content&gt;
+&lt;/appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>31348-32221</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>89 Stat. 641</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>89</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>94 Session 1</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Two sibling appropriations elements share identical heading "salaries and expenses"</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>TITLE II contains two sibling appropriations elements both with heading "Salaries and expenses" - one for Farmers Home Administration and one for Rural Electrification - that collapse to the same heading-derived Division UniqueKey. This is the same pattern covered by an existing approved extractor-code correction (active correction #5 from vol 78), and these rows will disambiguate automatically once that fix is generalized to vol 89.</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>&lt;appropriations&gt;
+&lt;heading&gt;salaries and expenses&lt;/heading&gt;
+&lt;content&gt;For necessary expenses of the Farmers Home Administration ...&lt;/content&gt;
+&lt;/appropriations&gt;
+&lt;appropriations&gt;
+&lt;heading&gt;salaries and expenses&lt;/heading&gt;
+&lt;content&gt;For administrative expenses to carry out the provisions of the Rural Electrification Act of 1936 ...&lt;/content&gt;
+&lt;/appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>32227-32724</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>89 Stat. 13</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>89</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>94 Session 1</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Public Law 94-7 silently dropped from the parsed output because its main contains quotedContent directly, no top-level section</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Extend the extractor's section walker to recognize "quotedContent" as a valid top-level body holder under "main" (alongside the existing section / part / title / bare-subsection branches). For PL 94-7, synthesize a single section row whose Text is the concatenated text of the quotedContent &gt; content node, carrying the joint-resolution long title through. Without this fix the validation report shows 207 distinct LawIdentifier vs 208 public pLaws in vol 89.</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>&lt;main&gt;
+&lt;longTitle&gt;
+&lt;docTitle&gt;Joint Resolution&lt;/docTitle&gt;
+&lt;officialTitle&gt;Making further continuing appropriations for the fiscal year 1975, and for other purposes.&lt;/officialTitle&gt;
+...
+&lt;/longTitle&gt;
+&lt;resolvingClause&gt;Resolved by the Senate and House of Representatives ...&lt;/resolvingClause&gt;
+&lt;quotedContent&gt;
+&lt;content class="inline"&gt;That clause, (c) of section 102 of the joint resolution of June 30, 1974 (Public Law 93–324, as amended by Public Law 93–448 and Public Law 93–570), is hereby further amended by striking out “February 28, 1975” and inserting in lieu thereof “June 30, 1975” ...&lt;/content&gt;
+&lt;/quotedContent&gt;
+&lt;action&gt;&lt;actionDescription&gt;Approved March 14, 1975.&lt;/actionDescription&gt;&lt;/action&gt;
+&lt;/main&gt;</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;quotedContent&gt;</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>2646-2659</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>90 Stat. 2479</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>90</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>94 Session 1</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Law number reported as 94–536 between Public Law 94–525 and Public Law 94–527</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Should be Public Law 94–526 — the volume's own front-matter index identifies this D.C. motor-vehicles act as Public Law 94–526 at 90 Stat. 2479, and the surrounding XML order requires 526 in this slot.</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>&lt;dc:title&gt;Public Law 94–536: To amend the Act establishing a code of law for the District of Columbia to prohibit the unauthorized use of a motor vehicle obtained under a written rental or other agreement.&lt;/dc:title&gt;
+&lt;dc:type&gt;Public Law&lt;/dc:type&gt;
+&lt;docNumber&gt;536&lt;/docNumber&gt;
+&lt;citableAs&gt;Public Law 94–536&lt;/citableAs&gt;
+&lt;citableAs&gt;90 Stat. 2479&lt;/citableAs&gt;</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;meta&gt;
+  &lt;docNumber&gt;
+   &lt;citableAs&gt;</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>139462-139555</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>90 Stat. 2481</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>90</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>94 Session 1</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Reviewed: gap — no correction needed</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Apparent sequence gap before Public Law 94–527 is an artefact of the preceding pLaw being misnumbered as 94–536 (true number 94–526). Public Law 94–527 itself is correctly numbered.</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>&lt;docNumber&gt;527&lt;/docNumber&gt;
+&lt;citableAs&gt;Public Law 94–527&lt;/citableAs&gt;
+&lt;citableAs&gt;90 Stat. 2481&lt;/citableAs&gt;
+&lt;officialTitle&gt;To amend the National Trails System Act (82 Stat. 919), and for other purposes.&lt;/officialTitle&gt;</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;meta&gt;
+  &lt;docNumber&gt;
+   &lt;citableAs&gt;</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>139562-139659</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>90 Stat. 2497</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>90</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>94 Session 1</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Reviewed: duplicate — no correction needed</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Apparent duplicate of law number 94–536 is an artefact of the earlier pLaw at 90 Stat. 2479 being misnumbered as 94–536 (true number 94–526). The pLaw at 90 Stat. 2497 (steamship United States floating-hotel act) is the legitimate Public Law 94–536.</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>&lt;docNumber&gt;536&lt;/docNumber&gt;
+&lt;citableAs&gt;Public Law 94–536&lt;/citableAs&gt;
+&lt;citableAs&gt;90 Stat. 2497&lt;/citableAs&gt;
+&lt;officialTitle&gt;To permit the steamship United Stares to be used as a floating hotel, and for other purposes.&lt;/officialTitle&gt;</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;meta&gt;
+  &lt;docNumber&gt;
+   &lt;citableAs&gt;</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>140489-140533</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>90 Stat. 2498</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>90</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>94 Session 1</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Reviewed: gap — no correction needed</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Apparent sequence gap before Public Law 94–537 is an artefact of the earlier pLaw at 90 Stat. 2479 being misnumbered as 94–536 (true number 94–526). Public Law 94–537 itself is correctly numbered.</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>&lt;docNumber&gt;537&lt;/docNumber&gt;
+&lt;citableAs&gt;Public Law 94–537&lt;/citableAs&gt;
+&lt;citableAs&gt;90 Stat. 2498&lt;/citableAs&gt;
+&lt;officialTitle&gt;To authorize the obligation and expenditure of funds to Implement for fiscal year 1877 the provisions of the Treaty of Friendship and Cooperation between the United States and Spain, signed at Madrid on January 24, 1970, and for other purposes.&lt;/officialTitle&gt;</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;meta&gt;
+  &lt;docNumber&gt;
+   &lt;citableAs&gt;</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>140540-140637</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>90 Stat. 383</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>90</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>94 Session 2</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Two sections both numbered Sec. 110 within the same Public Law</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>The second section labelled "Sec. 110." should be Sec. 116 — it sits between Sec. 115 and Sec. 117 in document order, so the "num" value should be 116.</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="110"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 110. &lt;/num&gt;
+&lt;content class="inline"&gt;For the purposes of sections 1079 and 1086 of title 10, United States Code, the period of July 1, 1976, through September 30, 1976, shall be considered a fiscal year...&lt;/content&gt;
+&lt;/section&gt;
+...
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="115"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 115. &lt;/num&gt;
+...
+&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="110"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 110. &lt;/num&gt;
+&lt;content class="inline"&gt;Notwithstanding the provisions of section 406(d) of the General Education Provisions Act (20 U.S.C. 1221 e–1 (d)), the report of the Assistant Secretary for the Department of Health, Education, and Welfare required by section 406(d) to be submitted in 1976 shall include a description of the activities of the National Center for Education Statistics during the period of July 1, 1976, through September 30, 1976.&lt;/content&gt;
+&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;
+&lt;num value="117"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 117. &lt;/num&gt;
+...</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>19272, 19330-19333</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>90 Stat. 597</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>90</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>94 Session 2</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Duplicate-heading sibling appropriations collapse to identical UniqueKey</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Two sibling "appropriations" elements under "Office of the Secretary / salaries and expenses" carry identical heading text — the second is a supplemental "additional amount" block with different content. Handled by the existing extractor convention that appends a sequential ordinal to duplicate-heading siblings; no XML change required.</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>&lt;appropriations&gt;
+ &lt;heading&gt;Office of the Secretary&lt;/heading&gt;
+ &lt;appropriations level="small"&gt;
+  &lt;heading&gt;salaries and expenses&lt;/heading&gt;
+  &lt;content&gt;Notwithstanding the limitation of funds available in the appropriation under this head in the Department of Transportation and Related Agencies Appropriation Act, 1975, to lease and maintain automobile parking facilities in the Nassif Building, payments of not to exceed $53,000 may be made out of any unobligated Departmental funds provided for fiscal year 1975 to pay the full court judgment awarded in June 1975 relating to such facilities.&lt;/content&gt;
+ &lt;/appropriations&gt;
+ &lt;appropriations level="small"&gt;
+  &lt;heading&gt;salaries and expenses&lt;/heading&gt;
+  &lt;content&gt;Of the amount provided under this head in the “Treasury, Postal Service, and General Government Appropriation Act, 1976”, $712,000 shall be available for expenses of travel...&lt;/content&gt;
+ &lt;/appropriations&gt;
+&lt;/appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;appropriations&gt;
+   &lt;appropriations&gt;</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>30427-32869</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>90 Stat. 1520</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>90</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>94 Session 2</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Two sections both numbered SEC. 801 within the same Public Law</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>The second section labelled "SEC. 801." should be SEC. 804 — it sits between SEC. 803 and SEC. 805 in TITLE VIII document order, so the "num" value should be 804.</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>&lt;section&gt;
+&lt;num value="801"&gt;SEC. 801. &lt;/num&gt;
+&lt;heading&gt;EXTENSION OF $100,000 LIMITATION ON USED PROPERTY FOR 4 YEARS.&lt;/heading&gt;
+&lt;content&gt;...Paragraph (2) of section 301(c) of the Tax Reduction Act of 1975 is amended...&lt;/content&gt;
+&lt;/section&gt;
+...
+&lt;section&gt;
+&lt;num value="803"&gt;SEC. 803. &lt;/num&gt;
+...
+&lt;/section&gt;
+&lt;section&gt;
+&lt;num value="801"&gt;SEC. 801. &lt;/num&gt;
+&lt;heading&gt;INVESTMENT CREDIT IN THE CASE OF MOVIE AND TELEVISION FILMS.&lt;/heading&gt;
+&lt;subsection&gt;&lt;num value="a"&gt;(a) &lt;/num&gt;&lt;heading&gt;Special Rules for Movie and Television Films.—&lt;/heading&gt;...&lt;/subsection&gt;
+&lt;/section&gt;
+&lt;section&gt;
+&lt;num value="805"&gt;SEC. 805. &lt;/num&gt;
+...</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;title&gt;
+   &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>83267, 83446, 83928, 84235</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>90 Stat. 2479</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>90</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>94 Session 1</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Duplicate LawIdentifier collapses two distinct Public Laws into one UniqueKey</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>The two rows sharing UniqueKey 094-536-000-000-000-000-000-S-000000000000001 are from two physically different pLaws — the D.C. motor-vehicles act at 90 Stat. 2479 (misnumbered as 94–536 in source XML; true number 94–526) and the legitimate steamship United States act at 90 Stat. 2497. Resolved by the same OCR fix that renumbers the 90 Stat. 2479 pLaw to Public Law 94–526.</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;meta&gt;
+  &lt;docNumber&gt;536&lt;/docNumber&gt;
+  &lt;citableAs&gt;Public Law 94–536&lt;/citableAs&gt;
+  &lt;citableAs&gt;90 Stat. 2479&lt;/citableAs&gt;
+  ...
+&lt;/pLaw&gt;
+&lt;pLaw&gt;
+ &lt;meta&gt;
+  &lt;docNumber&gt;536&lt;/docNumber&gt;
+  &lt;citableAs&gt;Public Law 94–536&lt;/citableAs&gt;
+  &lt;citableAs&gt;90 Stat. 2497&lt;/citableAs&gt;
+  ...
+&lt;/pLaw&gt;</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;meta&gt;
+  &lt;docNumber&gt;
+   &lt;citableAs&gt;</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>139462-139555, 140489-140533</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>90 Stat. 2732</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>90</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>94 Session 2</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Two sections both numbered Sec. 305 within the same Public Law</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>The second section labelled "Sec. 305." should be Sec. 306 — it sits between the first Sec. 305 and Sec. 307 in TITLE III document order, so the "num" value should be 306.</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>&lt;section class="firstIndent1 fontsize10"&gt;&lt;num value="304"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 304. &lt;/num&gt;...&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;&lt;num value="305"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 305. &lt;/num&gt;&lt;content class="inline"&gt;Section 2(c) of the Act of October 4, 1961 (75 Stat. 780), providing for the preservation and protection of certain lands in Prince Georges and Charles Counties, Maryland...&lt;/content&gt;&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;&lt;num value="305"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 305. &lt;/num&gt;&lt;content class="inline"&gt;Section 3 of the Act of August 31, 1964 (78 Stat. 749), authorizing the establishment of the SaintGaudens National Historic Site, New Hampshire, is amended by adding the following sentence...&lt;/content&gt;&lt;/section&gt;
+&lt;section class="firstIndent1 fontsize10"&gt;&lt;num value="307"&gt;&lt;inline class="smallCaps"&gt;Sec&lt;/inline&gt;. 307. &lt;/num&gt;...&lt;/section&gt;</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>&lt;pLaw&gt;
+ &lt;main&gt;
+  &lt;title&gt;
+   &lt;section&gt;</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>152762, 152773, 152776, 152779</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>